<commit_message>
Updated Cash Payment And Cash Receipt Functions
Updated Cash Payment And Cash Receipt Functions
</commit_message>
<xml_diff>
--- a/testdata/Financials.xlsx
+++ b/testdata/Financials.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="24" activeTab="26"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="53" activeTab="57"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2641" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2648" uniqueCount="357">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -1156,9 +1156,6 @@
   </si>
   <si>
     <t>TDS AMT</t>
-  </si>
-  <si>
-    <t>26550</t>
   </si>
 </sst>
 </file>
@@ -5738,11 +5735,11 @@
       <c r="Z2" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="AA2">
-        <v>0</v>
-      </c>
-      <c r="AB2">
-        <v>0</v>
+      <c r="AA2" t="s">
+        <v>310</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>310</v>
       </c>
       <c r="AC2">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
@@ -6418,11 +6415,11 @@
       <c r="Z2" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="AA2">
-        <v>0</v>
-      </c>
-      <c r="AB2">
-        <v>0</v>
+      <c r="AA2" t="s">
+        <v>310</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>310</v>
       </c>
       <c r="AC2">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
@@ -6495,11 +6492,11 @@
       <c r="Z3" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="AA3">
-        <v>0</v>
-      </c>
-      <c r="AB3">
-        <v>0</v>
+      <c r="AA3" t="s">
+        <v>310</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>310</v>
       </c>
       <c r="AC3">
         <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>
@@ -9354,10 +9351,10 @@
         <v>276</v>
       </c>
       <c r="AA2" t="s">
-        <v>357</v>
-      </c>
-      <c r="AB2">
-        <v>0</v>
+        <v>310</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>310</v>
       </c>
       <c r="AC2">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
@@ -9584,11 +9581,11 @@
       <c r="Z2" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="AA2">
-        <v>0</v>
-      </c>
-      <c r="AB2">
-        <v>0</v>
+      <c r="AA2" t="s">
+        <v>310</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>310</v>
       </c>
       <c r="AC2">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
@@ -9653,11 +9650,11 @@
       <c r="Z3" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="AA3">
-        <v>0</v>
-      </c>
-      <c r="AB3">
-        <v>0</v>
+      <c r="AA3" t="s">
+        <v>310</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>310</v>
       </c>
       <c r="AC3">
         <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>
@@ -10423,11 +10420,11 @@
       <c r="Z2" s="41" t="s">
         <v>276</v>
       </c>
-      <c r="AA2" t="s">
-        <v>310</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>310</v>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
       </c>
       <c r="AC2">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
@@ -10500,11 +10497,11 @@
       <c r="Z3" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="AA3" t="s">
-        <v>310</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>310</v>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
       </c>
       <c r="AC3" s="1">
         <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>

</xml_diff>

<commit_message>
Fixes For The Cash Payment Test Scenarios
Fixes For The Cash Payment Test Scenarios And Updated The Locators
</commit_message>
<xml_diff>
--- a/testdata/Financials.xlsx
+++ b/testdata/Financials.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="31" activeTab="33"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="85" activeTab="87"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -86,16 +86,16 @@
     <sheet name="TDS CPJournalADV" sheetId="125" r:id="rId77"/>
     <sheet name="CPJournalADV" sheetId="123" r:id="rId78"/>
     <sheet name="TDS CPAdvance" sheetId="124" r:id="rId79"/>
-    <sheet name="TDS CPJournalADVWithNewRef" sheetId="134" r:id="rId80"/>
-    <sheet name="TDS CPAdvanceWithNewRef" sheetId="133" r:id="rId81"/>
+    <sheet name="TDS CPAdvanceWithNewRef" sheetId="133" r:id="rId80"/>
+    <sheet name="TDS CPJournalADVWithNewRef" sheetId="134" r:id="rId81"/>
     <sheet name="TDS CPAdvanceMultiNewRef" sheetId="135" r:id="rId82"/>
     <sheet name="TDS CPJournalADVMultiNewref" sheetId="136" r:id="rId83"/>
     <sheet name="TDS CPAdvanceMulti" sheetId="130" r:id="rId84"/>
     <sheet name="TDS CPJournalADVMulti" sheetId="129" r:id="rId85"/>
     <sheet name="CPAdvanceMulti" sheetId="127" r:id="rId86"/>
     <sheet name="CPAdvanceWithNewRef" sheetId="132" r:id="rId87"/>
-    <sheet name="CPAdvance" sheetId="122" r:id="rId88"/>
-    <sheet name="CPJournalADVWithNewRef" sheetId="131" r:id="rId89"/>
+    <sheet name="CPJournalADVWithNewRef" sheetId="131" r:id="rId88"/>
+    <sheet name="CPAdvance" sheetId="122" r:id="rId89"/>
     <sheet name="BPJournalADVWithNewRef" sheetId="145" r:id="rId90"/>
     <sheet name="TDS BPJournalADVMultiNewref" sheetId="148" r:id="rId91"/>
     <sheet name="TDS BPJournalADVWithNewRef" sheetId="147" r:id="rId92"/>
@@ -181,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5523" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5487" uniqueCount="430">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -1321,9 +1321,6 @@
     <t>Purchase Order 2</t>
   </si>
   <si>
-    <t>CPC-10001</t>
-  </si>
-  <si>
     <t>194C</t>
   </si>
   <si>
@@ -1378,9 +1375,6 @@
     <t>Charges</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>10000</t>
   </si>
   <si>
@@ -1475,6 +1469,9 @@
   </si>
   <si>
     <t>UNRELIZED GAIN/LOSS</t>
+  </si>
+  <si>
+    <t>1000</t>
   </si>
 </sst>
 </file>
@@ -1482,19 +1479,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="34">
+  <fonts count="33">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1824,21 +1814,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1847,25 +1837,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyBorder="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="2" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
@@ -1877,10 +1867,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1890,86 +1880,83 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
@@ -1978,31 +1965,34 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
@@ -2011,25 +2001,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
@@ -2041,10 +2028,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
@@ -2071,7 +2058,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -7500,7 +7487,7 @@
         <v>309</v>
       </c>
       <c r="AD1" s="64" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="2" spans="1:30">
@@ -7956,7 +7943,7 @@
       </c>
       <c r="I2" s="47">
         <f>ROUND(SUM(ROUND(G2,2)+ROUND(H2,2))*K1,2)</f>
-        <v>11000</v>
+        <v>8500</v>
       </c>
       <c r="J2" s="59">
         <v>0</v>
@@ -8006,7 +7993,7 @@
       </c>
       <c r="J3" s="59">
         <f>ROUND(SUM(ROUND(G3,2)+ROUND(H3,2))*K1,2)</f>
-        <v>11000</v>
+        <v>8500</v>
       </c>
     </row>
   </sheetData>
@@ -14195,14 +14182,14 @@
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="76" t="s">
+      <c r="B2" s="75" t="s">
+        <v>398</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>400</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>402</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>281</v>
@@ -14210,7 +14197,7 @@
       <c r="F2" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="G2" s="75" t="s">
+      <c r="G2" s="74" t="s">
         <v>339</v>
       </c>
       <c r="H2" s="22" t="s">
@@ -14441,7 +14428,7 @@
       <c r="F2" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="G2" s="75" t="s">
+      <c r="G2" s="74" t="s">
         <v>339</v>
       </c>
       <c r="H2" s="22" t="s">
@@ -14820,19 +14807,19 @@
         <v>329</v>
       </c>
       <c r="AD1" s="64" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AE1" s="64" t="s">
+        <v>389</v>
+      </c>
+      <c r="AF1" s="64" t="s">
         <v>390</v>
       </c>
-      <c r="AF1" s="64" t="s">
+      <c r="AG1" s="64" t="s">
         <v>391</v>
       </c>
-      <c r="AG1" s="64" t="s">
+      <c r="AH1" s="64" t="s">
         <v>392</v>
-      </c>
-      <c r="AH1" s="64" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:34">
@@ -14912,7 +14899,7 @@
         <v>0</v>
       </c>
       <c r="AD2" t="s" s="0">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AE2" s="0">
         <v>1000000029</v>
@@ -14933,12 +14920,12 @@
       <c r="A3" s="24">
         <v>2</v>
       </c>
-      <c r="B3" s="68" t="s">
+      <c r="B3" s="67" t="s">
         <v>349</v>
       </c>
       <c r="C3" s="24"/>
       <c r="D3" s="24" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E3" s="24"/>
       <c r="F3" s="1" t="s">
@@ -14947,12 +14934,12 @@
       <c r="G3" s="24" t="s">
         <v>339</v>
       </c>
-      <c r="H3" s="66"/>
+      <c r="H3" s="65"/>
       <c r="I3" s="24"/>
       <c r="J3" s="24" t="s">
         <v>303</v>
       </c>
-      <c r="K3" s="69" t="s">
+      <c r="K3" s="68" t="s">
         <v>207</v>
       </c>
       <c r="L3" t="s" s="0">
@@ -15160,7 +15147,7 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="70" t="s">
+      <c r="B3" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C3" s="1">
@@ -15187,8 +15174,8 @@
       <c r="K3" s="24"/>
       <c r="L3" s="24"/>
       <c r="M3" s="24"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
       <c r="Q3" s="24"/>
       <c r="R3" s="24"/>
       <c r="S3" s="24"/>
@@ -15366,19 +15353,19 @@
         <v>309</v>
       </c>
       <c r="AD1" s="64" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AE1" s="64" t="s">
+        <v>389</v>
+      </c>
+      <c r="AF1" s="64" t="s">
         <v>390</v>
       </c>
-      <c r="AF1" s="64" t="s">
+      <c r="AG1" s="64" t="s">
         <v>391</v>
       </c>
-      <c r="AG1" s="64" t="s">
+      <c r="AH1" s="64" t="s">
         <v>392</v>
-      </c>
-      <c r="AH1" s="64" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:34">
@@ -15395,7 +15382,7 @@
         <v>375</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>316</v>
@@ -15458,7 +15445,7 @@
         <v>221.25</v>
       </c>
       <c r="AD2" t="s" s="0">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AE2" s="0">
         <v>1000000029</v>
@@ -15479,22 +15466,22 @@
       <c r="A3" s="41">
         <v>2</v>
       </c>
-      <c r="B3" s="71" t="s">
+      <c r="B3" s="70" t="s">
+        <v>381</v>
+      </c>
+      <c r="C3" s="41" t="s">
         <v>382</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="D3" s="41" t="s">
         <v>383</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="E3" s="41" t="s">
         <v>384</v>
-      </c>
-      <c r="E3" s="41" t="s">
-        <v>385</v>
       </c>
       <c r="F3" s="41" t="s">
         <v>316</v>
       </c>
-      <c r="G3" s="72" t="s">
+      <c r="G3" s="71" t="s">
         <v>339</v>
       </c>
       <c r="H3" s="44" t="s">
@@ -15552,7 +15539,7 @@
         <v>221.25</v>
       </c>
       <c r="AD3" t="s" s="0">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="AE3" s="0">
         <v>1000000047</v>
@@ -15577,7 +15564,7 @@
         <v>349</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>349</v>
@@ -15666,14 +15653,14 @@
       <c r="A5" s="14">
         <v>4</v>
       </c>
-      <c r="B5" s="73" t="s">
+      <c r="B5" s="72" t="s">
+        <v>387</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>386</v>
+      </c>
+      <c r="D5" s="73" t="s">
         <v>388</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>387</v>
-      </c>
-      <c r="D5" s="74" t="s">
-        <v>389</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="14" t="s">
@@ -15975,7 +15962,7 @@
         <v>2000000100</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -16014,7 +16001,7 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="70" t="s">
+      <c r="B4" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C4" s="1">
@@ -16041,8 +16028,8 @@
       <c r="K4" s="24"/>
       <c r="L4" s="24"/>
       <c r="M4" s="24"/>
-      <c r="O4" s="67"/>
-      <c r="P4" s="67"/>
+      <c r="O4" s="66"/>
+      <c r="P4" s="66"/>
       <c r="Q4" s="24"/>
       <c r="R4" s="24"/>
       <c r="S4" s="24"/>
@@ -16060,14 +16047,14 @@
       <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="B5" s="70" t="s">
+      <c r="B5" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C5" s="1">
         <v>1000000047</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -16087,8 +16074,8 @@
       <c r="K5" s="24"/>
       <c r="L5" s="24"/>
       <c r="M5" s="24"/>
-      <c r="O5" s="67"/>
-      <c r="P5" s="67"/>
+      <c r="O5" s="66"/>
+      <c r="P5" s="66"/>
       <c r="Q5" s="24"/>
       <c r="R5" s="24"/>
       <c r="S5" s="24"/>
@@ -16398,7 +16385,7 @@
         <v>2000000118</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -16522,10 +16509,10 @@
         <v>255</v>
       </c>
       <c r="E1" s="56" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="F1" s="56" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="G1" s="37" t="s">
         <v>256</v>
@@ -16591,45 +16578,45 @@
         <v>306</v>
       </c>
       <c r="AB1" s="64" t="s">
+        <v>407</v>
+      </c>
+      <c r="AC1" s="64" t="s">
+        <v>408</v>
+      </c>
+      <c r="AD1" s="64" t="s">
         <v>409</v>
       </c>
-      <c r="AC1" s="64" t="s">
+      <c r="AE1" s="64" t="s">
         <v>410</v>
       </c>
-      <c r="AD1" s="64" t="s">
+      <c r="AF1" s="64" t="s">
+        <v>413</v>
+      </c>
+      <c r="AG1" s="64" t="s">
+        <v>414</v>
+      </c>
+      <c r="AH1" s="64" t="s">
         <v>411</v>
       </c>
-      <c r="AE1" s="64" t="s">
+      <c r="AI1" s="64" t="s">
         <v>412</v>
-      </c>
-      <c r="AF1" s="64" t="s">
-        <v>415</v>
-      </c>
-      <c r="AG1" s="64" t="s">
-        <v>416</v>
-      </c>
-      <c r="AH1" s="64" t="s">
-        <v>413</v>
-      </c>
-      <c r="AI1" s="64" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="2" spans="1:35">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="77" t="s">
-        <v>407</v>
+      <c r="B2" s="76" t="s">
+        <v>405</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>405</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>281</v>
@@ -16685,16 +16672,16 @@
         <v>303</v>
       </c>
       <c r="AB2" t="s" s="0">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AC2" t="s" s="0">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AD2" t="s" s="0">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="AE2" t="s" s="0">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="AF2" s="0">
         <f>ROUND(AD2-AB2,2)</f>
@@ -16717,17 +16704,17 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="77" t="s">
-        <v>408</v>
+      <c r="B3" s="76" t="s">
+        <v>406</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>406</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>281</v>
@@ -16783,16 +16770,16 @@
         <v>303</v>
       </c>
       <c r="AB3" t="s" s="0">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AC3" t="s" s="0">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AD3" t="s" s="0">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="AE3" t="s" s="0">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="AF3" s="0">
         <f>ROUND(AD3-AB3,2)</f>
@@ -16921,10 +16908,10 @@
         <v>255</v>
       </c>
       <c r="E1" s="56" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="F1" s="56" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="G1" s="37" t="s">
         <v>256</v>
@@ -16990,45 +16977,45 @@
         <v>306</v>
       </c>
       <c r="AB1" s="64" t="s">
+        <v>407</v>
+      </c>
+      <c r="AC1" s="64" t="s">
+        <v>408</v>
+      </c>
+      <c r="AD1" s="64" t="s">
         <v>409</v>
       </c>
-      <c r="AC1" s="64" t="s">
+      <c r="AE1" s="64" t="s">
         <v>410</v>
       </c>
-      <c r="AD1" s="64" t="s">
+      <c r="AF1" s="64" t="s">
+        <v>413</v>
+      </c>
+      <c r="AG1" s="64" t="s">
+        <v>414</v>
+      </c>
+      <c r="AH1" s="64" t="s">
         <v>411</v>
       </c>
-      <c r="AE1" s="64" t="s">
+      <c r="AI1" s="64" t="s">
         <v>412</v>
-      </c>
-      <c r="AF1" s="64" t="s">
-        <v>415</v>
-      </c>
-      <c r="AG1" s="64" t="s">
-        <v>416</v>
-      </c>
-      <c r="AH1" s="64" t="s">
-        <v>413</v>
-      </c>
-      <c r="AI1" s="64" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="2" spans="1:35">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="76" t="s">
+      <c r="B2" s="75" t="s">
+        <v>398</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>402</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>281</v>
@@ -17084,16 +17071,16 @@
         <v>303</v>
       </c>
       <c r="AB2" t="s" s="0">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="AC2" t="s" s="0">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="AD2" t="s" s="0">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="AE2" t="s" s="0">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="AF2" s="0">
         <f>ROUND(AD2-AB2,2)</f>
@@ -17116,17 +17103,17 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="78" t="s">
-        <v>423</v>
+      <c r="B3" s="77" t="s">
+        <v>421</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>420</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>422</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>281</v>
@@ -17182,16 +17169,16 @@
         <v>303</v>
       </c>
       <c r="AB3" t="s" s="0">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="AC3" t="s" s="0">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="AD3" t="s" s="0">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="AE3" t="s" s="0">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="AF3" s="0">
         <f>ROUND(AD3-AB3,2)</f>
@@ -19501,7 +19488,7 @@
       <c r="J2" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="K2" s="79" t="s">
+      <c r="K2" s="78" t="s">
         <v>209</v>
       </c>
       <c r="L2" t="s" s="0">
@@ -19763,7 +19750,7 @@
         <v>303</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="AB2" t="s" s="0">
         <v>310</v>
@@ -19777,14 +19764,14 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="80" t="s">
+      <c r="B3" s="79" t="s">
+        <v>424</v>
+      </c>
+      <c r="C3" s="79" t="s">
+        <v>425</v>
+      </c>
+      <c r="D3" s="79" t="s">
         <v>426</v>
-      </c>
-      <c r="C3" s="80" t="s">
-        <v>427</v>
-      </c>
-      <c r="D3" s="80" t="s">
-        <v>428</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>334</v>
@@ -19843,7 +19830,7 @@
         <v>310</v>
       </c>
       <c r="AB3" t="s" s="0">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="AC3" s="0">
         <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>
@@ -20070,10 +20057,10 @@
         <v>303</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="AB2" t="s" s="0">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="AC2" s="0">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
@@ -20084,14 +20071,14 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="80" t="s">
+      <c r="B3" s="79" t="s">
+        <v>424</v>
+      </c>
+      <c r="C3" s="79" t="s">
+        <v>425</v>
+      </c>
+      <c r="D3" s="79" t="s">
         <v>426</v>
-      </c>
-      <c r="C3" s="80" t="s">
-        <v>427</v>
-      </c>
-      <c r="D3" s="80" t="s">
-        <v>428</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>334</v>
@@ -20147,10 +20134,10 @@
         <v>303</v>
       </c>
       <c r="AA3" t="s" s="0">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="AB3" t="s" s="0">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="AC3" s="0">
         <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>
@@ -20541,14 +20528,14 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="80" t="s">
+      <c r="B3" s="79" t="s">
+        <v>424</v>
+      </c>
+      <c r="C3" s="79" t="s">
+        <v>425</v>
+      </c>
+      <c r="D3" s="79" t="s">
         <v>426</v>
-      </c>
-      <c r="C3" s="80" t="s">
-        <v>427</v>
-      </c>
-      <c r="D3" s="80" t="s">
-        <v>428</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>334</v>
@@ -20783,8 +20770,8 @@
       <c r="C3" s="1">
         <v>2000000124</v>
       </c>
-      <c r="D3" s="80" t="s">
-        <v>426</v>
+      <c r="D3" s="79" t="s">
+        <v>424</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -20959,8 +20946,8 @@
       <c r="C3" s="1">
         <v>2000000124</v>
       </c>
-      <c r="D3" s="80" t="s">
-        <v>426</v>
+      <c r="D3" s="79" t="s">
+        <v>424</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -21162,8 +21149,8 @@
       <c r="C3" s="1">
         <v>2000000124</v>
       </c>
-      <c r="D3" s="80" t="s">
-        <v>426</v>
+      <c r="D3" s="79" t="s">
+        <v>424</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -21701,7 +21688,7 @@
         <v>5050606001</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -21712,7 +21699,7 @@
       <c r="H4" s="0">
         <v>0</v>
       </c>
-      <c r="I4" s="81">
+      <c r="I4" s="80">
         <v>0</v>
       </c>
       <c r="J4" s="59">
@@ -30916,7 +30903,7 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" t="s" s="0">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="H2" t="s" s="0">
         <v>310</v>
@@ -31339,7 +31326,7 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="70" t="s">
+      <c r="B3" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C3" s="1">
@@ -31366,8 +31353,8 @@
       <c r="K3" s="24"/>
       <c r="L3" s="24"/>
       <c r="M3" s="24"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
       <c r="Q3" s="24"/>
       <c r="R3" s="24"/>
       <c r="S3" s="24"/>
@@ -31516,7 +31503,7 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" t="s" s="0">
-        <v>381</v>
+        <v>310</v>
       </c>
       <c r="H2" t="s" s="0">
         <v>310</v>
@@ -31562,7 +31549,7 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" t="s" s="0">
-        <v>381</v>
+        <v>310</v>
       </c>
       <c r="H3" t="s" s="0">
         <v>310</v>
@@ -31583,7 +31570,7 @@
 
 <file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC4"/>
+  <dimension ref="A1:AH4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
@@ -31614,9 +31601,13 @@
     <col min="26" max="26" bestFit="true" customWidth="true" width="15.0"/>
     <col min="27" max="28" bestFit="true" customWidth="true" width="14.7109375"/>
     <col min="29" max="29" bestFit="true" customWidth="true" width="25.0"/>
+    <col min="31" max="31" customWidth="true" width="16.28515625"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="14.0"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="23.140625"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="16.5703125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29">
+    <row r="1" spans="1:34">
       <c r="A1" s="37" t="s">
         <v>253</v>
       </c>
@@ -31704,8 +31695,23 @@
       <c r="AC1" s="40" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="2" spans="1:29">
+      <c r="AD1" s="64" t="s">
+        <v>385</v>
+      </c>
+      <c r="AE1" s="64" t="s">
+        <v>389</v>
+      </c>
+      <c r="AF1" s="64" t="s">
+        <v>390</v>
+      </c>
+      <c r="AG1" s="64" t="s">
+        <v>391</v>
+      </c>
+      <c r="AH1" s="64" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="2" spans="1:34">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -31724,8 +31730,8 @@
       <c r="F2" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="G2" s="65" t="s">
-        <v>379</v>
+      <c r="G2" s="24" t="s">
+        <v>339</v>
       </c>
       <c r="H2" s="22" t="s">
         <v>275</v>
@@ -31744,16 +31750,17 @@
       </c>
       <c r="M2" s="38">
         <f>ROUND(SUM(AA2+AB2+I2),2)</f>
-        <v>0</v>
+        <v>221.25</v>
       </c>
       <c r="N2" s="38">
         <f>AC2</f>
-        <v>0</v>
+        <v>221.25</v>
       </c>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1">
-        <v>0</v>
+        <f>AC2</f>
+        <v>221.25</v>
       </c>
       <c r="R2" s="1"/>
       <c r="S2" s="1"/>
@@ -31778,19 +31785,36 @@
       </c>
       <c r="AC2" s="0">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29">
+        <v>221.25</v>
+      </c>
+      <c r="AD2" t="s" s="0">
+        <v>379</v>
+      </c>
+      <c r="AE2" s="0">
+        <v>1000000029</v>
+      </c>
+      <c r="AF2" s="0">
+        <v>1</v>
+      </c>
+      <c r="AG2" s="0">
+        <f>AC2</f>
+        <v>221.25</v>
+      </c>
+      <c r="AH2" s="0">
+        <f>ROUND(AC2*AF2%,2)</f>
+        <v>2.21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:34">
       <c r="A3" s="24">
         <v>2</v>
       </c>
-      <c r="B3" s="68" t="s">
+      <c r="B3" s="67" t="s">
         <v>349</v>
       </c>
       <c r="C3" s="24"/>
       <c r="D3" s="24" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E3" s="24"/>
       <c r="F3" s="1" t="s">
@@ -31799,12 +31823,12 @@
       <c r="G3" s="24" t="s">
         <v>339</v>
       </c>
-      <c r="H3" s="66"/>
+      <c r="H3" s="65"/>
       <c r="I3" s="24"/>
       <c r="J3" s="24" t="s">
         <v>303</v>
       </c>
-      <c r="K3" s="69" t="s">
+      <c r="K3" s="68" t="s">
         <v>207</v>
       </c>
       <c r="L3" t="s" s="0">
@@ -31812,11 +31836,11 @@
       </c>
       <c r="M3" s="38">
         <f>AC3</f>
-        <v>0</v>
+        <v>2.21</v>
       </c>
       <c r="N3" s="38">
         <f>AC3</f>
-        <v>0</v>
+        <v>2.21</v>
       </c>
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
@@ -31846,21 +31870,30 @@
       </c>
       <c r="AC3" s="0">
         <f>ROUND(AA2*1%,2)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:29">
+        <v>2.21</v>
+      </c>
+      <c r="AF3" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34">
       <c r="M4" s="0">
         <f>SUM(M2)</f>
-        <v>0</v>
+        <v>221.25</v>
       </c>
       <c r="N4" s="0">
         <f>SUM(N2)</f>
-        <v>0</v>
+        <v>221.25</v>
       </c>
       <c r="Q4" s="0">
         <f>SUM(Q2)</f>
-        <v>0</v>
+        <v>221.25</v>
       </c>
       <c r="AA4" t="s" s="0">
         <v>310</v>
@@ -31870,7 +31903,7 @@
       </c>
       <c r="AC4" s="0">
         <f>SUM(AC2)</f>
-        <v>0</v>
+        <v>221.25</v>
       </c>
     </row>
   </sheetData>
@@ -31986,217 +32019,6 @@
 </file>
 
 <file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="23.0"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="28.7109375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="33.42578125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="28.7109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="18.42578125"/>
-    <col min="7" max="8" customWidth="true" width="18.42578125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="14.5703125"/>
-    <col min="10" max="10" customWidth="true" width="17.42578125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="21.5703125"/>
-    <col min="13" max="13" customWidth="true" width="21.5703125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="16.0"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="16.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="16.5703125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="20.0"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:31">
-      <c r="A1" s="56" t="s">
-        <v>253</v>
-      </c>
-      <c r="B1" s="56" t="s">
-        <v>183</v>
-      </c>
-      <c r="C1" s="56" t="s">
-        <v>352</v>
-      </c>
-      <c r="D1" s="56" t="s">
-        <v>254</v>
-      </c>
-      <c r="E1" s="56" t="s">
-        <v>353</v>
-      </c>
-      <c r="F1" s="56" t="s">
-        <v>257</v>
-      </c>
-      <c r="G1" s="56" t="s">
-        <v>357</v>
-      </c>
-      <c r="H1" s="56" t="s">
-        <v>358</v>
-      </c>
-      <c r="I1" s="56" t="s">
-        <v>354</v>
-      </c>
-      <c r="J1" s="56" t="s">
-        <v>355</v>
-      </c>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
-      <c r="P1" s="37"/>
-      <c r="Q1" s="37"/>
-      <c r="R1" s="37"/>
-      <c r="S1" s="37"/>
-      <c r="T1" s="37"/>
-      <c r="U1" s="37"/>
-      <c r="V1" s="37"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="46"/>
-      <c r="Y1" s="46"/>
-      <c r="Z1" s="40"/>
-      <c r="AA1" s="40"/>
-      <c r="AB1" s="37"/>
-      <c r="AC1" s="40"/>
-      <c r="AD1" s="40"/>
-      <c r="AE1" s="40"/>
-    </row>
-    <row r="2" spans="1:31">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="58" t="s">
-        <v>191</v>
-      </c>
-      <c r="C2" s="1">
-        <v>2000000099</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="I2" s="47">
-        <f>ROUND(SUM(G2+H2),2)</f>
-        <v>0</v>
-      </c>
-      <c r="J2" s="59">
-        <v>0</v>
-      </c>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="O2" s="38"/>
-      <c r="P2" s="38"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
-      <c r="W2" s="1"/>
-      <c r="X2" s="1"/>
-      <c r="Y2" s="1"/>
-      <c r="Z2" s="1"/>
-      <c r="AA2" s="1"/>
-      <c r="AB2" s="1"/>
-    </row>
-    <row r="3" spans="1:31">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="70" t="s">
-        <v>191</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1000000029</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>349</v>
-      </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="H3" s="0">
-        <v>0</v>
-      </c>
-      <c r="I3" s="47">
-        <v>0</v>
-      </c>
-      <c r="J3" s="59">
-        <f>ROUND(I2*1%,2)</f>
-        <v>0</v>
-      </c>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="24"/>
-      <c r="R3" s="24"/>
-      <c r="S3" s="24"/>
-      <c r="T3" s="24"/>
-      <c r="U3" s="24"/>
-      <c r="V3" s="24"/>
-      <c r="W3" s="24"/>
-      <c r="X3" s="24"/>
-      <c r="Y3" s="24"/>
-      <c r="Z3" s="24"/>
-      <c r="AA3" s="24"/>
-      <c r="AB3" s="24"/>
-    </row>
-    <row r="4" spans="1:31">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="58" t="s">
-        <v>191</v>
-      </c>
-      <c r="C4" s="1">
-        <v>1000000028</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="H4" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="I4" s="59">
-        <v>0</v>
-      </c>
-      <c r="J4" s="59">
-        <f>ROUND(I2-J3,2)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" ht="9" customHeight="1"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AH4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -32324,19 +32146,19 @@
         <v>329</v>
       </c>
       <c r="AD1" s="64" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AE1" s="64" t="s">
+        <v>389</v>
+      </c>
+      <c r="AF1" s="64" t="s">
         <v>390</v>
       </c>
-      <c r="AF1" s="64" t="s">
+      <c r="AG1" s="64" t="s">
         <v>391</v>
       </c>
-      <c r="AG1" s="64" t="s">
+      <c r="AH1" s="64" t="s">
         <v>392</v>
-      </c>
-      <c r="AH1" s="64" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:34">
@@ -32416,7 +32238,7 @@
         <v>1000</v>
       </c>
       <c r="AD2" t="s" s="0">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AE2" s="0">
         <v>1000000029</v>
@@ -32441,7 +32263,7 @@
         <v>349</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>349</v>
@@ -32453,12 +32275,12 @@
       <c r="G3" s="24" t="s">
         <v>339</v>
       </c>
-      <c r="H3" s="66"/>
+      <c r="H3" s="65"/>
       <c r="I3" s="24"/>
       <c r="J3" s="24" t="s">
         <v>303</v>
       </c>
-      <c r="K3" s="69" t="s">
+      <c r="K3" s="68" t="s">
         <v>207</v>
       </c>
       <c r="L3" t="s" s="0">
@@ -32550,6 +32372,217 @@
         <v>990</v>
       </c>
     </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AE9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="23.0"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="28.7109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="33.42578125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="28.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="18.42578125"/>
+    <col min="7" max="8" customWidth="true" width="18.42578125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="14.5703125"/>
+    <col min="10" max="10" customWidth="true" width="17.42578125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="21.5703125"/>
+    <col min="13" max="13" customWidth="true" width="21.5703125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="16.0"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="16.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="16.5703125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="20.0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31">
+      <c r="A1" s="56" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" s="56" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1" s="56" t="s">
+        <v>352</v>
+      </c>
+      <c r="D1" s="56" t="s">
+        <v>254</v>
+      </c>
+      <c r="E1" s="56" t="s">
+        <v>353</v>
+      </c>
+      <c r="F1" s="56" t="s">
+        <v>257</v>
+      </c>
+      <c r="G1" s="56" t="s">
+        <v>357</v>
+      </c>
+      <c r="H1" s="56" t="s">
+        <v>358</v>
+      </c>
+      <c r="I1" s="56" t="s">
+        <v>354</v>
+      </c>
+      <c r="J1" s="56" t="s">
+        <v>355</v>
+      </c>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="37"/>
+      <c r="T1" s="37"/>
+      <c r="U1" s="37"/>
+      <c r="V1" s="37"/>
+      <c r="W1" s="46"/>
+      <c r="X1" s="46"/>
+      <c r="Y1" s="46"/>
+      <c r="Z1" s="40"/>
+      <c r="AA1" s="40"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="40"/>
+      <c r="AD1" s="40"/>
+      <c r="AE1" s="40"/>
+    </row>
+    <row r="2" spans="1:31">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="58" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2000000099</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="I2" s="47">
+        <f>ROUND(SUM(G2+H2),2)</f>
+        <v>0</v>
+      </c>
+      <c r="J2" s="59">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="O2" s="38"/>
+      <c r="P2" s="38"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+    </row>
+    <row r="3" spans="1:31">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="69" t="s">
+        <v>191</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1000000029</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="H3" s="0">
+        <v>0</v>
+      </c>
+      <c r="I3" s="47">
+        <v>0</v>
+      </c>
+      <c r="J3" s="59">
+        <f>ROUND(I2*1%,2)</f>
+        <v>0</v>
+      </c>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="24"/>
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
+      <c r="Q3" s="24"/>
+      <c r="R3" s="24"/>
+      <c r="S3" s="24"/>
+      <c r="T3" s="24"/>
+      <c r="U3" s="24"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="24"/>
+      <c r="X3" s="24"/>
+      <c r="Y3" s="24"/>
+      <c r="Z3" s="24"/>
+      <c r="AA3" s="24"/>
+      <c r="AB3" s="24"/>
+    </row>
+    <row r="4" spans="1:31">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="58" t="s">
+        <v>191</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1000000028</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="I4" s="59">
+        <v>0</v>
+      </c>
+      <c r="J4" s="59">
+        <f>ROUND(I2-J3,2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" ht="9" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -32684,19 +32717,19 @@
         <v>309</v>
       </c>
       <c r="AD1" s="64" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AE1" s="64" t="s">
+        <v>389</v>
+      </c>
+      <c r="AF1" s="64" t="s">
         <v>390</v>
       </c>
-      <c r="AF1" s="64" t="s">
+      <c r="AG1" s="64" t="s">
         <v>391</v>
       </c>
-      <c r="AG1" s="64" t="s">
+      <c r="AH1" s="64" t="s">
         <v>392</v>
-      </c>
-      <c r="AH1" s="64" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:34">
@@ -32713,7 +32746,7 @@
         <v>375</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>316</v>
@@ -32776,7 +32809,7 @@
         <v>10000</v>
       </c>
       <c r="AD2" t="s" s="0">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AE2" s="0">
         <v>1000000029</v>
@@ -32797,26 +32830,26 @@
       <c r="A3" s="41">
         <v>2</v>
       </c>
-      <c r="B3" s="71" t="s">
+      <c r="B3" s="70" t="s">
+        <v>381</v>
+      </c>
+      <c r="C3" s="41" t="s">
         <v>382</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="D3" s="41" t="s">
         <v>383</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="E3" s="41" t="s">
         <v>384</v>
-      </c>
-      <c r="E3" s="41" t="s">
-        <v>385</v>
       </c>
       <c r="F3" s="41" t="s">
         <v>316</v>
       </c>
-      <c r="G3" s="72" t="s">
+      <c r="G3" s="71" t="s">
         <v>339</v>
       </c>
       <c r="H3" s="44" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I3" s="41">
         <v>10000</v>
@@ -32870,7 +32903,7 @@
         <v>10000</v>
       </c>
       <c r="AD3" t="s" s="0">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="AE3" s="0">
         <v>1000000047</v>
@@ -32895,7 +32928,7 @@
         <v>349</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>349</v>
@@ -32908,7 +32941,7 @@
         <v>339</v>
       </c>
       <c r="H4" s="44" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="I4" s="1">
         <v>0</v>
@@ -32984,14 +33017,14 @@
       <c r="A5" s="14">
         <v>4</v>
       </c>
-      <c r="B5" s="73" t="s">
+      <c r="B5" s="72" t="s">
+        <v>387</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>386</v>
+      </c>
+      <c r="D5" s="73" t="s">
         <v>388</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>387</v>
-      </c>
-      <c r="D5" s="74" t="s">
-        <v>389</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="14" t="s">
@@ -33001,7 +33034,7 @@
         <v>339</v>
       </c>
       <c r="H5" s="44" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I5" s="1">
         <v>0</v>
@@ -33203,7 +33236,7 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" t="s" s="0">
-        <v>399</v>
+        <v>310</v>
       </c>
       <c r="H2" t="s" s="0">
         <v>310</v>
@@ -33244,12 +33277,12 @@
         <v>2000000100</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" t="s" s="0">
-        <v>399</v>
+        <v>310</v>
       </c>
       <c r="H3" t="s" s="0">
         <v>310</v>
@@ -33283,7 +33316,7 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="70" t="s">
+      <c r="B4" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C4" s="1">
@@ -33310,8 +33343,8 @@
       <c r="K4" s="24"/>
       <c r="L4" s="24"/>
       <c r="M4" s="24"/>
-      <c r="O4" s="67"/>
-      <c r="P4" s="67"/>
+      <c r="O4" s="66"/>
+      <c r="P4" s="66"/>
       <c r="Q4" s="24"/>
       <c r="R4" s="24"/>
       <c r="S4" s="24"/>
@@ -33329,14 +33362,14 @@
       <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="B5" s="70" t="s">
+      <c r="B5" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C5" s="1">
         <v>1000000047</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -33356,8 +33389,8 @@
       <c r="K5" s="24"/>
       <c r="L5" s="24"/>
       <c r="M5" s="24"/>
-      <c r="O5" s="67"/>
-      <c r="P5" s="67"/>
+      <c r="O5" s="66"/>
+      <c r="P5" s="66"/>
       <c r="Q5" s="24"/>
       <c r="R5" s="24"/>
       <c r="S5" s="24"/>
@@ -33535,19 +33568,19 @@
         <v>309</v>
       </c>
       <c r="AD1" s="64" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AE1" s="64" t="s">
+        <v>389</v>
+      </c>
+      <c r="AF1" s="64" t="s">
         <v>390</v>
       </c>
-      <c r="AF1" s="64" t="s">
+      <c r="AG1" s="64" t="s">
         <v>391</v>
       </c>
-      <c r="AG1" s="64" t="s">
+      <c r="AH1" s="64" t="s">
         <v>392</v>
-      </c>
-      <c r="AH1" s="64" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:34">
@@ -33564,7 +33597,7 @@
         <v>375</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>316</v>
@@ -33627,7 +33660,7 @@
         <v>0</v>
       </c>
       <c r="AD2" t="s" s="0">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AE2" s="0">
         <v>1000000029</v>
@@ -33648,22 +33681,22 @@
       <c r="A3" s="41">
         <v>2</v>
       </c>
-      <c r="B3" s="71" t="s">
+      <c r="B3" s="70" t="s">
+        <v>381</v>
+      </c>
+      <c r="C3" s="41" t="s">
         <v>382</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="D3" s="41" t="s">
         <v>383</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="E3" s="41" t="s">
         <v>384</v>
-      </c>
-      <c r="E3" s="41" t="s">
-        <v>385</v>
       </c>
       <c r="F3" s="41" t="s">
         <v>316</v>
       </c>
-      <c r="G3" s="72" t="s">
+      <c r="G3" s="71" t="s">
         <v>339</v>
       </c>
       <c r="H3" s="44" t="s">
@@ -33721,7 +33754,7 @@
         <v>0</v>
       </c>
       <c r="AD3" t="s" s="0">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="AE3" s="0">
         <v>1000000047</v>
@@ -33746,7 +33779,7 @@
         <v>349</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>349</v>
@@ -33835,14 +33868,14 @@
       <c r="A5" s="14">
         <v>4</v>
       </c>
-      <c r="B5" s="73" t="s">
+      <c r="B5" s="72" t="s">
+        <v>387</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>386</v>
+      </c>
+      <c r="D5" s="73" t="s">
         <v>388</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>387</v>
-      </c>
-      <c r="D5" s="74" t="s">
-        <v>389</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="14" t="s">
@@ -34095,7 +34128,7 @@
         <v>2000000100</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -34134,7 +34167,7 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="70" t="s">
+      <c r="B4" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C4" s="1">
@@ -34161,8 +34194,8 @@
       <c r="K4" s="24"/>
       <c r="L4" s="24"/>
       <c r="M4" s="24"/>
-      <c r="O4" s="67"/>
-      <c r="P4" s="67"/>
+      <c r="O4" s="66"/>
+      <c r="P4" s="66"/>
       <c r="Q4" s="24"/>
       <c r="R4" s="24"/>
       <c r="S4" s="24"/>
@@ -34180,14 +34213,14 @@
       <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="B5" s="70" t="s">
+      <c r="B5" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C5" s="1">
         <v>1000000047</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -34207,8 +34240,8 @@
       <c r="K5" s="24"/>
       <c r="L5" s="24"/>
       <c r="M5" s="24"/>
-      <c r="O5" s="67"/>
-      <c r="P5" s="67"/>
+      <c r="O5" s="66"/>
+      <c r="P5" s="66"/>
       <c r="Q5" s="24"/>
       <c r="R5" s="24"/>
       <c r="S5" s="24"/>
@@ -34396,7 +34429,7 @@
         <v>375</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>316</v>
@@ -34449,7 +34482,7 @@
         <v>303</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AB2" t="s" s="0">
         <v>310</v>
@@ -34464,16 +34497,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="63" t="s">
+        <v>381</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>384</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>385</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>316</v>
@@ -34526,7 +34559,7 @@
         <v>303</v>
       </c>
       <c r="AA3" t="s" s="0">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AB3" s="0">
         <v>0</v>
@@ -34688,7 +34721,7 @@
         <v>329</v>
       </c>
       <c r="AD1" s="64" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="2" spans="1:30">
@@ -34768,7 +34801,7 @@
         <v>1000</v>
       </c>
       <c r="AD2" t="s" s="0">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="3" spans="1:30">
@@ -34802,6 +34835,170 @@
 </file>
 
 <file path=xl/worksheets/sheet88.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AE3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="23.0"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="28.7109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="33.42578125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="28.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="18.42578125"/>
+    <col min="7" max="8" customWidth="true" width="18.42578125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="14.5703125"/>
+    <col min="10" max="10" customWidth="true" width="17.42578125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="21.5703125"/>
+    <col min="13" max="13" customWidth="true" width="21.5703125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="16.0"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="16.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="16.5703125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="20.0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31">
+      <c r="A1" s="56" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" s="56" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1" s="56" t="s">
+        <v>352</v>
+      </c>
+      <c r="D1" s="56" t="s">
+        <v>254</v>
+      </c>
+      <c r="E1" s="56" t="s">
+        <v>353</v>
+      </c>
+      <c r="F1" s="56" t="s">
+        <v>257</v>
+      </c>
+      <c r="G1" s="56" t="s">
+        <v>357</v>
+      </c>
+      <c r="H1" s="56" t="s">
+        <v>358</v>
+      </c>
+      <c r="I1" s="56" t="s">
+        <v>354</v>
+      </c>
+      <c r="J1" s="56" t="s">
+        <v>355</v>
+      </c>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="37"/>
+      <c r="T1" s="37"/>
+      <c r="U1" s="37"/>
+      <c r="V1" s="37"/>
+      <c r="W1" s="46"/>
+      <c r="X1" s="46"/>
+      <c r="Y1" s="46"/>
+      <c r="Z1" s="40"/>
+      <c r="AA1" s="40"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="40"/>
+      <c r="AD1" s="40"/>
+      <c r="AE1" s="40"/>
+    </row>
+    <row r="2" spans="1:31">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="58" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2000000099</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="H2" s="0">
+        <v>0</v>
+      </c>
+      <c r="I2" s="47">
+        <f>ROUND(SUM(G2+H2),2)</f>
+        <v>1000</v>
+      </c>
+      <c r="J2" s="59">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="O2" s="38"/>
+      <c r="P2" s="38"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+    </row>
+    <row r="3" spans="1:31">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="58" t="s">
+        <v>191</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1000000028</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="H3" s="0">
+        <v>0</v>
+      </c>
+      <c r="I3" s="59">
+        <v>0</v>
+      </c>
+      <c r="J3" s="59">
+        <f>ROUND(SUM(G3+H3),2)</f>
+        <v>1000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet89.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AC3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -34944,8 +35141,8 @@
       <c r="F2" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="G2" s="65" t="s">
-        <v>379</v>
+      <c r="G2" s="47" t="s">
+        <v>339</v>
       </c>
       <c r="H2" s="22" t="s">
         <v>275</v>
@@ -34992,7 +35189,7 @@
         <v>303</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>381</v>
+        <v>310</v>
       </c>
       <c r="AB2" t="s" s="0">
         <v>310</v>
@@ -35023,170 +35220,6 @@
       </c>
       <c r="AC3" s="0">
         <f>SUM(AC2)</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet89.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="23.0"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="28.7109375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="33.42578125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="28.7109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="18.42578125"/>
-    <col min="7" max="8" customWidth="true" width="18.42578125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="14.5703125"/>
-    <col min="10" max="10" customWidth="true" width="17.42578125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="21.5703125"/>
-    <col min="13" max="13" customWidth="true" width="21.5703125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="16.0"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="16.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="16.5703125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="20.0"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:31">
-      <c r="A1" s="56" t="s">
-        <v>253</v>
-      </c>
-      <c r="B1" s="56" t="s">
-        <v>183</v>
-      </c>
-      <c r="C1" s="56" t="s">
-        <v>352</v>
-      </c>
-      <c r="D1" s="56" t="s">
-        <v>254</v>
-      </c>
-      <c r="E1" s="56" t="s">
-        <v>353</v>
-      </c>
-      <c r="F1" s="56" t="s">
-        <v>257</v>
-      </c>
-      <c r="G1" s="56" t="s">
-        <v>357</v>
-      </c>
-      <c r="H1" s="56" t="s">
-        <v>358</v>
-      </c>
-      <c r="I1" s="56" t="s">
-        <v>354</v>
-      </c>
-      <c r="J1" s="56" t="s">
-        <v>355</v>
-      </c>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
-      <c r="P1" s="37"/>
-      <c r="Q1" s="37"/>
-      <c r="R1" s="37"/>
-      <c r="S1" s="37"/>
-      <c r="T1" s="37"/>
-      <c r="U1" s="37"/>
-      <c r="V1" s="37"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="46"/>
-      <c r="Y1" s="46"/>
-      <c r="Z1" s="40"/>
-      <c r="AA1" s="40"/>
-      <c r="AB1" s="37"/>
-      <c r="AC1" s="40"/>
-      <c r="AD1" s="40"/>
-      <c r="AE1" s="40"/>
-    </row>
-    <row r="2" spans="1:31">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="58" t="s">
-        <v>191</v>
-      </c>
-      <c r="C2" s="1">
-        <v>2000000099</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" t="s" s="0">
-        <v>398</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="I2" s="47">
-        <f>ROUND(SUM(G2+H2),2)</f>
-        <v>0</v>
-      </c>
-      <c r="J2" s="59">
-        <v>0</v>
-      </c>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="O2" s="38"/>
-      <c r="P2" s="38"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
-      <c r="W2" s="1"/>
-      <c r="X2" s="1"/>
-      <c r="Y2" s="1"/>
-      <c r="Z2" s="1"/>
-      <c r="AA2" s="1"/>
-      <c r="AB2" s="1"/>
-    </row>
-    <row r="3" spans="1:31">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="58" t="s">
-        <v>191</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1000000028</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" t="s" s="0">
-        <v>398</v>
-      </c>
-      <c r="H3" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="I3" s="59">
-        <v>0</v>
-      </c>
-      <c r="J3" s="59">
-        <f>ROUND(SUM(G3+H3),2)</f>
         <v>0</v>
       </c>
     </row>
@@ -36443,7 +36476,7 @@
         <v>2000000100</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -36482,7 +36515,7 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="70" t="s">
+      <c r="B4" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C4" s="1">
@@ -36509,8 +36542,8 @@
       <c r="K4" s="24"/>
       <c r="L4" s="24"/>
       <c r="M4" s="24"/>
-      <c r="O4" s="67"/>
-      <c r="P4" s="67"/>
+      <c r="O4" s="66"/>
+      <c r="P4" s="66"/>
       <c r="Q4" s="24"/>
       <c r="R4" s="24"/>
       <c r="S4" s="24"/>
@@ -36528,14 +36561,14 @@
       <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="B5" s="70" t="s">
+      <c r="B5" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C5" s="1">
         <v>1000000047</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -36555,8 +36588,8 @@
       <c r="K5" s="24"/>
       <c r="L5" s="24"/>
       <c r="M5" s="24"/>
-      <c r="O5" s="67"/>
-      <c r="P5" s="67"/>
+      <c r="O5" s="66"/>
+      <c r="P5" s="66"/>
       <c r="Q5" s="24"/>
       <c r="R5" s="24"/>
       <c r="S5" s="24"/>
@@ -36739,7 +36772,7 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="70" t="s">
+      <c r="B3" s="69" t="s">
         <v>191</v>
       </c>
       <c r="C3" s="1">
@@ -36766,8 +36799,8 @@
       <c r="K3" s="24"/>
       <c r="L3" s="24"/>
       <c r="M3" s="24"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
       <c r="Q3" s="24"/>
       <c r="R3" s="24"/>
       <c r="S3" s="24"/>

</xml_diff>

<commit_message>
Updated New Sheet Name For The Direct GRN
Updated New Sheet Name For The Direct GRN
</commit_message>
<xml_diff>
--- a/testdata/Financials.xlsx
+++ b/testdata/Financials.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="85" activeTab="87"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="123" activeTab="123"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -181,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5487" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5496" uniqueCount="429">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -1375,9 +1375,6 @@
     <t>Charges</t>
   </si>
   <si>
-    <t>10000</t>
-  </si>
-  <si>
     <t>MAERSK SEALAND(AP)</t>
   </si>
   <si>
@@ -1471,7 +1468,7 @@
     <t>UNRELIZED GAIN/LOSS</t>
   </si>
   <si>
-    <t>1000</t>
+    <t>26550</t>
   </si>
 </sst>
 </file>
@@ -3224,8 +3221,8 @@
       <c r="G2" t="s" s="0">
         <v>310</v>
       </c>
-      <c r="H2" s="0">
-        <v>0</v>
+      <c r="H2" t="s" s="0">
+        <v>310</v>
       </c>
       <c r="I2" s="47">
         <f>ROUND(SUM(G2+H2),2)</f>
@@ -3270,8 +3267,8 @@
       <c r="G3" t="s" s="0">
         <v>310</v>
       </c>
-      <c r="H3" s="0">
-        <v>0</v>
+      <c r="H3" t="s" s="0">
+        <v>310</v>
       </c>
       <c r="I3" s="59">
         <v>0</v>
@@ -8330,7 +8327,7 @@
       </c>
       <c r="N2" s="38">
         <f>AC2</f>
-        <v>26550</v>
+        <v>0</v>
       </c>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
@@ -8361,7 +8358,7 @@
       </c>
       <c r="AC2" s="0">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
-        <v>26550</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:29">
@@ -8371,7 +8368,7 @@
       </c>
       <c r="N3" s="0">
         <f>SUM(N2)</f>
-        <v>26550</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="0">
         <f>SUM(Q2)</f>
@@ -8385,7 +8382,7 @@
       </c>
       <c r="AC3" s="0">
         <f>SUM(AC2)</f>
-        <v>26550</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -8586,10 +8583,10 @@
         <v>276</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>310</v>
+        <v>428</v>
       </c>
       <c r="AB2" t="s" s="0">
-        <v>310</v>
+        <v>428</v>
       </c>
       <c r="AC2" s="0">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
@@ -8655,10 +8652,10 @@
         <v>276</v>
       </c>
       <c r="AA3" t="s" s="0">
-        <v>310</v>
+        <v>428</v>
       </c>
       <c r="AB3" t="s" s="0">
-        <v>310</v>
+        <v>428</v>
       </c>
       <c r="AC3" s="0">
         <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>
@@ -14183,13 +14180,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="75" t="s">
+        <v>397</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>399</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>400</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>281</v>
@@ -16385,7 +16382,7 @@
         <v>2000000118</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -16509,10 +16506,10 @@
         <v>255</v>
       </c>
       <c r="E1" s="56" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F1" s="56" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G1" s="37" t="s">
         <v>256</v>
@@ -16578,28 +16575,28 @@
         <v>306</v>
       </c>
       <c r="AB1" s="64" t="s">
+        <v>406</v>
+      </c>
+      <c r="AC1" s="64" t="s">
         <v>407</v>
       </c>
-      <c r="AC1" s="64" t="s">
+      <c r="AD1" s="64" t="s">
         <v>408</v>
       </c>
-      <c r="AD1" s="64" t="s">
+      <c r="AE1" s="64" t="s">
         <v>409</v>
       </c>
-      <c r="AE1" s="64" t="s">
+      <c r="AF1" s="64" t="s">
+        <v>412</v>
+      </c>
+      <c r="AG1" s="64" t="s">
+        <v>413</v>
+      </c>
+      <c r="AH1" s="64" t="s">
         <v>410</v>
       </c>
-      <c r="AF1" s="64" t="s">
-        <v>413</v>
-      </c>
-      <c r="AG1" s="64" t="s">
-        <v>414</v>
-      </c>
-      <c r="AH1" s="64" t="s">
+      <c r="AI1" s="64" t="s">
         <v>411</v>
-      </c>
-      <c r="AI1" s="64" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="2" spans="1:35">
@@ -16607,13 +16604,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="76" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>384</v>
@@ -16678,10 +16675,10 @@
         <v>380</v>
       </c>
       <c r="AD2" t="s" s="0">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="AE2" t="s" s="0">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="AF2" s="0">
         <f>ROUND(AD2-AB2,2)</f>
@@ -16705,13 +16702,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="76" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>384</v>
@@ -16776,10 +16773,10 @@
         <v>380</v>
       </c>
       <c r="AD3" t="s" s="0">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="AE3" t="s" s="0">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="AF3" s="0">
         <f>ROUND(AD3-AB3,2)</f>
@@ -16908,10 +16905,10 @@
         <v>255</v>
       </c>
       <c r="E1" s="56" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F1" s="56" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G1" s="37" t="s">
         <v>256</v>
@@ -16977,28 +16974,28 @@
         <v>306</v>
       </c>
       <c r="AB1" s="64" t="s">
+        <v>406</v>
+      </c>
+      <c r="AC1" s="64" t="s">
         <v>407</v>
       </c>
-      <c r="AC1" s="64" t="s">
+      <c r="AD1" s="64" t="s">
         <v>408</v>
       </c>
-      <c r="AD1" s="64" t="s">
+      <c r="AE1" s="64" t="s">
         <v>409</v>
       </c>
-      <c r="AE1" s="64" t="s">
+      <c r="AF1" s="64" t="s">
+        <v>412</v>
+      </c>
+      <c r="AG1" s="64" t="s">
+        <v>413</v>
+      </c>
+      <c r="AH1" s="64" t="s">
         <v>410</v>
       </c>
-      <c r="AF1" s="64" t="s">
-        <v>413</v>
-      </c>
-      <c r="AG1" s="64" t="s">
-        <v>414</v>
-      </c>
-      <c r="AH1" s="64" t="s">
+      <c r="AI1" s="64" t="s">
         <v>411</v>
-      </c>
-      <c r="AI1" s="64" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="2" spans="1:35">
@@ -17006,16 +17003,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="75" t="s">
+        <v>397</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>400</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>281</v>
@@ -17071,16 +17068,16 @@
         <v>303</v>
       </c>
       <c r="AB2" t="s" s="0">
+        <v>421</v>
+      </c>
+      <c r="AC2" t="s" s="0">
+        <v>421</v>
+      </c>
+      <c r="AD2" t="s" s="0">
         <v>422</v>
       </c>
-      <c r="AC2" t="s" s="0">
+      <c r="AE2" t="s" s="0">
         <v>422</v>
-      </c>
-      <c r="AD2" t="s" s="0">
-        <v>423</v>
-      </c>
-      <c r="AE2" t="s" s="0">
-        <v>423</v>
       </c>
       <c r="AF2" s="0">
         <f>ROUND(AD2-AB2,2)</f>
@@ -17104,16 +17101,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="77" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>419</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>420</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>281</v>
@@ -17169,16 +17166,16 @@
         <v>303</v>
       </c>
       <c r="AB3" t="s" s="0">
+        <v>421</v>
+      </c>
+      <c r="AC3" t="s" s="0">
+        <v>421</v>
+      </c>
+      <c r="AD3" t="s" s="0">
         <v>422</v>
       </c>
-      <c r="AC3" t="s" s="0">
+      <c r="AE3" t="s" s="0">
         <v>422</v>
-      </c>
-      <c r="AD3" t="s" s="0">
-        <v>423</v>
-      </c>
-      <c r="AE3" t="s" s="0">
-        <v>423</v>
       </c>
       <c r="AF3" s="0">
         <f>ROUND(AD3-AB3,2)</f>
@@ -19750,7 +19747,7 @@
         <v>303</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="AB2" t="s" s="0">
         <v>310</v>
@@ -19765,13 +19762,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="79" t="s">
+        <v>423</v>
+      </c>
+      <c r="C3" s="79" t="s">
         <v>424</v>
       </c>
-      <c r="C3" s="79" t="s">
+      <c r="D3" s="79" t="s">
         <v>425</v>
-      </c>
-      <c r="D3" s="79" t="s">
-        <v>426</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>334</v>
@@ -19830,7 +19827,7 @@
         <v>310</v>
       </c>
       <c r="AB3" t="s" s="0">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="AC3" s="0">
         <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>
@@ -20057,10 +20054,10 @@
         <v>303</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="AB2" t="s" s="0">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="AC2" s="0">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
@@ -20072,13 +20069,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="79" t="s">
+        <v>423</v>
+      </c>
+      <c r="C3" s="79" t="s">
         <v>424</v>
       </c>
-      <c r="C3" s="79" t="s">
+      <c r="D3" s="79" t="s">
         <v>425</v>
-      </c>
-      <c r="D3" s="79" t="s">
-        <v>426</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>334</v>
@@ -20134,10 +20131,10 @@
         <v>303</v>
       </c>
       <c r="AA3" t="s" s="0">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="AB3" t="s" s="0">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="AC3" s="0">
         <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>
@@ -20529,13 +20526,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="79" t="s">
+        <v>423</v>
+      </c>
+      <c r="C3" s="79" t="s">
         <v>424</v>
       </c>
-      <c r="C3" s="79" t="s">
+      <c r="D3" s="79" t="s">
         <v>425</v>
-      </c>
-      <c r="D3" s="79" t="s">
-        <v>426</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>334</v>
@@ -20771,7 +20768,7 @@
         <v>2000000124</v>
       </c>
       <c r="D3" s="79" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -20947,7 +20944,7 @@
         <v>2000000124</v>
       </c>
       <c r="D3" s="79" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -21150,7 +21147,7 @@
         <v>2000000124</v>
       </c>
       <c r="D3" s="79" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -21688,7 +21685,7 @@
         <v>5050606001</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -30903,7 +30900,7 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" t="s" s="0">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="H2" t="s" s="0">
         <v>310</v>

</xml_diff>

<commit_message>
Updated The Fixes In Bank Payment And Cash Payment
Updated The Fixes In Bank Payment And Cash Payment Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/Financials.xlsx
+++ b/testdata/Financials.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="123" activeTab="123"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="136" activeTab="137"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -144,11 +144,11 @@
     <sheet name="BankPaymentChargesINR" sheetId="112" r:id="rId135"/>
     <sheet name="BankPaymentCharges" sheetId="65" r:id="rId136"/>
     <sheet name="BankPaymentExpGST" sheetId="63" r:id="rId137"/>
-    <sheet name="BankPaymentExpUSD" sheetId="103" r:id="rId138"/>
-    <sheet name="BankPaymentExp" sheetId="62" r:id="rId139"/>
-    <sheet name="BankReceiptRevExp" sheetId="58" r:id="rId140"/>
-    <sheet name="BankPaymentExpTDS" sheetId="66" r:id="rId141"/>
-    <sheet name="BankPaymentExpGSTTDS" sheetId="67" r:id="rId142"/>
+    <sheet name="BankPaymentExpGSTTDS" sheetId="67" r:id="rId138"/>
+    <sheet name="BankPaymentExpUSD" sheetId="103" r:id="rId139"/>
+    <sheet name="BankPaymentExp" sheetId="62" r:id="rId140"/>
+    <sheet name="BankReceiptRevExp" sheetId="58" r:id="rId141"/>
+    <sheet name="BankPaymentExpTDS" sheetId="66" r:id="rId142"/>
     <sheet name="BankPaymentPDC" sheetId="61" r:id="rId143"/>
     <sheet name="BPAdvanceUSD" sheetId="161" r:id="rId144"/>
     <sheet name="BPAdvance" sheetId="154" r:id="rId145"/>
@@ -181,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5496" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5626" uniqueCount="429">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -11988,6 +11988,435 @@
 
 <file path=xl/worksheets/sheet138.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr codeName="Sheet108"/>
+  <dimension ref="A1:AL4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="26.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="9.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.7109375"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.85546875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="7.140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="9.28515625"/>
+    <col min="8" max="8" customWidth="true" width="17.42578125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="12.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="7.0"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="8.140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.5703125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="16.5703125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="5.5703125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="5.42578125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="5.0"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="6.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="8.42578125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="27" max="28" bestFit="true" customWidth="true" width="8.85546875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="20.0"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="12.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="3.0"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="19.42578125"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="5.140625"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" width="16.0"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="14.0"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" width="23.140625"/>
+    <col min="38" max="38" bestFit="true" customWidth="true" width="16.5703125"/>
+    <col min="39" max="39" bestFit="true" customWidth="true" width="19.42578125"/>
+    <col min="40" max="40" bestFit="true" customWidth="true" width="17.7109375"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:38">
+      <c r="A1" s="37" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" s="37" t="s">
+        <v>254</v>
+      </c>
+      <c r="C1" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="D1" s="37" t="s">
+        <v>255</v>
+      </c>
+      <c r="E1" s="37" t="s">
+        <v>279</v>
+      </c>
+      <c r="F1" s="37" t="s">
+        <v>256</v>
+      </c>
+      <c r="G1" s="37" t="s">
+        <v>257</v>
+      </c>
+      <c r="H1" s="37" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1" s="37" t="s">
+        <v>258</v>
+      </c>
+      <c r="J1" s="37" t="s">
+        <v>305</v>
+      </c>
+      <c r="K1" s="37" t="s">
+        <v>261</v>
+      </c>
+      <c r="L1" s="37" t="s">
+        <v>262</v>
+      </c>
+      <c r="M1" s="37" t="s">
+        <v>273</v>
+      </c>
+      <c r="N1" s="37" t="s">
+        <v>263</v>
+      </c>
+      <c r="O1" s="37" t="s">
+        <v>264</v>
+      </c>
+      <c r="P1" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="Q1" s="37" t="s">
+        <v>266</v>
+      </c>
+      <c r="R1" s="37" t="s">
+        <v>267</v>
+      </c>
+      <c r="S1" s="37" t="s">
+        <v>268</v>
+      </c>
+      <c r="T1" s="37" t="s">
+        <v>269</v>
+      </c>
+      <c r="U1" s="46" t="s">
+        <v>270</v>
+      </c>
+      <c r="V1" s="46" t="s">
+        <v>271</v>
+      </c>
+      <c r="W1" s="46" t="s">
+        <v>272</v>
+      </c>
+      <c r="X1" s="40" t="s">
+        <v>304</v>
+      </c>
+      <c r="Y1" s="40" t="s">
+        <v>204</v>
+      </c>
+      <c r="Z1" s="37" t="s">
+        <v>306</v>
+      </c>
+      <c r="AA1" s="40" t="s">
+        <v>307</v>
+      </c>
+      <c r="AB1" s="40" t="s">
+        <v>308</v>
+      </c>
+      <c r="AC1" s="40" t="s">
+        <v>309</v>
+      </c>
+      <c r="AD1" s="40" t="s">
+        <v>336</v>
+      </c>
+      <c r="AE1" s="0">
+        <v>1</v>
+      </c>
+      <c r="AF1" s="55" t="s">
+        <v>348</v>
+      </c>
+      <c r="AG1" s="54" t="s">
+        <v>347</v>
+      </c>
+      <c r="AH1" s="64" t="s">
+        <v>385</v>
+      </c>
+      <c r="AI1" s="64" t="s">
+        <v>389</v>
+      </c>
+      <c r="AJ1" s="64" t="s">
+        <v>390</v>
+      </c>
+      <c r="AK1" s="64" t="s">
+        <v>391</v>
+      </c>
+      <c r="AL1" s="64" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="2" spans="1:38">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="48" t="s">
+        <v>340</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G2" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="H2" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="I2" s="1">
+        <v>1000</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>319</v>
+      </c>
+      <c r="M2" s="38">
+        <f>ROUND(SUM(AA2+AB2+I2),2)</f>
+        <v>1000</v>
+      </c>
+      <c r="N2" s="38">
+        <f>ROUND(SUM(AA2+AB2+I2),2)</f>
+        <v>1000</v>
+      </c>
+      <c r="O2" s="1">
+        <v>88363222</v>
+      </c>
+      <c r="P2" s="53">
+        <v>0.18</v>
+      </c>
+      <c r="Q2" s="1">
+        <f>M2</f>
+        <v>1000</v>
+      </c>
+      <c r="R2" s="1">
+        <f>IF(OR($AE$1=1,$AE$1=4),ROUND((Q2*P2)/2,2),0)</f>
+        <v>90</v>
+      </c>
+      <c r="S2" s="1">
+        <f>IF($AE$1=1,ROUND(((Q2*P2)/2),2),0)</f>
+        <v>90</v>
+      </c>
+      <c r="T2" s="1">
+        <f>IF($AE$1=2,ROUND(((Q2*P2)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="U2" s="1">
+        <f>IF($AE$1=4,ROUND(((Q2*P2)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="V2" s="1">
+        <v>0</v>
+      </c>
+      <c r="W2" s="1">
+        <v>0</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="AA2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="AB2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="AC2" s="0">
+        <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)+R2+S2+T2+U2+W2),2)</f>
+        <v>1180</v>
+      </c>
+      <c r="AD2" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="AE2" s="0">
+        <v>34</v>
+      </c>
+      <c r="AF2" t="s" s="0">
+        <v>345</v>
+      </c>
+      <c r="AG2" t="s" s="0">
+        <v>346</v>
+      </c>
+      <c r="AH2" t="s" s="0">
+        <v>379</v>
+      </c>
+      <c r="AI2" s="0">
+        <v>1000000029</v>
+      </c>
+      <c r="AJ2" s="0">
+        <v>1</v>
+      </c>
+      <c r="AK2" s="0">
+        <f>I2</f>
+        <v>1000</v>
+      </c>
+      <c r="AL2" s="0">
+        <f>ROUND(M2*AJ2%,2)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:38">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="57" t="s">
+        <v>349</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G3" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>342</v>
+      </c>
+      <c r="I3" s="1">
+        <f>AK2</f>
+        <v>1000</v>
+      </c>
+      <c r="J3" s="14" t="s">
+        <v>303</v>
+      </c>
+      <c r="K3" s="14" t="s">
+        <v>207</v>
+      </c>
+      <c r="L3" s="1">
+        <v>1</v>
+      </c>
+      <c r="M3" s="38">
+        <f>M2*1%</f>
+        <v>10</v>
+      </c>
+      <c r="N3" s="38">
+        <f>M2*1%</f>
+        <v>10</v>
+      </c>
+      <c r="O3" s="1"/>
+      <c r="P3" s="53">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>0</v>
+      </c>
+      <c r="R3" s="1">
+        <f>IF(OR($AE$1=1,$AE$1=4),ROUND((Q3*P3)/2,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="S3" s="1">
+        <f>IF($AE$1=1,ROUND(((Q3*P3)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="T3" s="1">
+        <f>IF($AE$1=2,ROUND(((Q3*P3)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="U3" s="1">
+        <f>IF($AE$1=4,ROUND(((Q3*P3)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="V3" s="1">
+        <v>0</v>
+      </c>
+      <c r="W3" s="1">
+        <v>0</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="AA3" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="AB3" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="AC3" s="1">
+        <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)+R3+S3+T3+U3+W3),2)</f>
+        <v>1000</v>
+      </c>
+      <c r="AD3" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="AE3" s="1"/>
+      <c r="AF3" s="1"/>
+      <c r="AG3" s="1"/>
+      <c r="AH3" s="1"/>
+      <c r="AI3" s="1"/>
+      <c r="AJ3" s="1"/>
+      <c r="AK3" s="1"/>
+    </row>
+    <row r="4" spans="1:38">
+      <c r="I4" s="0">
+        <f>SUM(I2:I2)</f>
+        <v>1000</v>
+      </c>
+      <c r="M4" s="0">
+        <f>SUM(M2+R2+S2+T2+U2+W2)-M3</f>
+        <v>1170</v>
+      </c>
+      <c r="N4" s="0">
+        <f>SUM(N2+R2+S2+T2+U2+W2)-N3</f>
+        <v>1170</v>
+      </c>
+      <c r="Q4" s="0">
+        <f>SUM(Q2:Q2)</f>
+        <v>1000</v>
+      </c>
+      <c r="R4" s="0">
+        <f>SUM(R2:R2)</f>
+        <v>90</v>
+      </c>
+      <c r="S4" s="0">
+        <f>SUM(S2:S2)</f>
+        <v>90</v>
+      </c>
+      <c r="T4" s="0">
+        <f>SUM(T2:T2)</f>
+        <v>0</v>
+      </c>
+      <c r="U4" s="0">
+        <f>SUM(U2:U2)</f>
+        <v>0</v>
+      </c>
+      <c r="AC4" s="0">
+        <f>AC2-AC3</f>
+        <v>180</v>
+      </c>
+      <c r="AD4" t="s" s="0">
+        <v>337</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet139.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet104"/>
   <dimension ref="A1:AG3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -12271,7 +12700,88 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet139.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr codeName="Sheet14"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="24.85546875"/>
+    <col min="2" max="2" customWidth="true" width="11.5703125"/>
+    <col min="3" max="3" customWidth="true" width="9.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.28515625"/>
+    <col min="5" max="5" customWidth="true" width="19.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.28515625"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="36" t="s">
+        <v>250</v>
+      </c>
+      <c r="E1" s="36" t="s">
+        <v>246</v>
+      </c>
+      <c r="F1" s="36" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" s="1">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="F2" s="0">
+        <f>ROUND(C2*E2,2)</f>
+        <v>847.48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C3" s="1">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>248</v>
+      </c>
+      <c r="F3" s="0">
+        <f>ROUND(C3*E3,2)</f>
+        <v>159.26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet140.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet105"/>
   <dimension ref="A1:AG3"/>
@@ -12556,88 +13066,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr codeName="Sheet14"/>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="24.85546875"/>
-    <col min="2" max="2" customWidth="true" width="11.5703125"/>
-    <col min="3" max="3" customWidth="true" width="9.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="19.28515625"/>
-    <col min="5" max="5" customWidth="true" width="19.28515625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.28515625"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="36" t="s">
-        <v>250</v>
-      </c>
-      <c r="E1" s="36" t="s">
-        <v>246</v>
-      </c>
-      <c r="F1" s="36" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="C2" s="1">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>249</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>251</v>
-      </c>
-      <c r="F2" s="0">
-        <f>ROUND(C2*E2,2)</f>
-        <v>847.48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="C3" s="1">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>252</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>248</v>
-      </c>
-      <c r="F3" s="0">
-        <f>ROUND(C3*E3,2)</f>
-        <v>159.26</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet140.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet141.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet106"/>
   <dimension ref="A1:AG4"/>
@@ -13025,7 +13454,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet141.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet142.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet107"/>
   <dimension ref="A1:AI4"/>
@@ -13404,401 +13833,6 @@
       </c>
       <c r="U4" s="0">
         <f>SUM(U2:U3)</f>
-        <v>0</v>
-      </c>
-      <c r="AC4" s="0">
-        <f>AC2-AC3</f>
-        <v>1170</v>
-      </c>
-      <c r="AD4" t="s" s="0">
-        <v>337</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet142.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr codeName="Sheet108"/>
-  <dimension ref="A1:AI4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="26.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="28.7109375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="28.7109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="18.42578125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="14.5703125"/>
-    <col min="8" max="8" customWidth="true" width="17.42578125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="21.5703125"/>
-    <col min="11" max="11" customWidth="true" width="21.5703125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="16.0"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="16.7109375"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="16.5703125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="20.0"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="12.0"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="19.42578125"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="17.7109375"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:35">
-      <c r="A1" s="37" t="s">
-        <v>253</v>
-      </c>
-      <c r="B1" s="37" t="s">
-        <v>254</v>
-      </c>
-      <c r="C1" s="37" t="s">
-        <v>287</v>
-      </c>
-      <c r="D1" s="37" t="s">
-        <v>255</v>
-      </c>
-      <c r="E1" s="37" t="s">
-        <v>279</v>
-      </c>
-      <c r="F1" s="37" t="s">
-        <v>256</v>
-      </c>
-      <c r="G1" s="37" t="s">
-        <v>257</v>
-      </c>
-      <c r="H1" s="37" t="s">
-        <v>259</v>
-      </c>
-      <c r="I1" s="37" t="s">
-        <v>258</v>
-      </c>
-      <c r="J1" s="37" t="s">
-        <v>305</v>
-      </c>
-      <c r="K1" s="37" t="s">
-        <v>261</v>
-      </c>
-      <c r="L1" s="37" t="s">
-        <v>262</v>
-      </c>
-      <c r="M1" s="37" t="s">
-        <v>273</v>
-      </c>
-      <c r="N1" s="37" t="s">
-        <v>263</v>
-      </c>
-      <c r="O1" s="37" t="s">
-        <v>264</v>
-      </c>
-      <c r="P1" s="37" t="s">
-        <v>265</v>
-      </c>
-      <c r="Q1" s="37" t="s">
-        <v>266</v>
-      </c>
-      <c r="R1" s="37" t="s">
-        <v>267</v>
-      </c>
-      <c r="S1" s="37" t="s">
-        <v>268</v>
-      </c>
-      <c r="T1" s="37" t="s">
-        <v>269</v>
-      </c>
-      <c r="U1" s="46" t="s">
-        <v>270</v>
-      </c>
-      <c r="V1" s="46" t="s">
-        <v>271</v>
-      </c>
-      <c r="W1" s="46" t="s">
-        <v>272</v>
-      </c>
-      <c r="X1" s="40" t="s">
-        <v>304</v>
-      </c>
-      <c r="Y1" s="40" t="s">
-        <v>204</v>
-      </c>
-      <c r="Z1" s="37" t="s">
-        <v>306</v>
-      </c>
-      <c r="AA1" s="40" t="s">
-        <v>307</v>
-      </c>
-      <c r="AB1" s="40" t="s">
-        <v>308</v>
-      </c>
-      <c r="AC1" s="40" t="s">
-        <v>309</v>
-      </c>
-      <c r="AD1" s="40" t="s">
-        <v>336</v>
-      </c>
-      <c r="AE1" s="0">
-        <v>1</v>
-      </c>
-      <c r="AF1" s="55" t="s">
-        <v>348</v>
-      </c>
-      <c r="AG1" s="54" t="s">
-        <v>347</v>
-      </c>
-      <c r="AH1" s="56" t="s">
-        <v>350</v>
-      </c>
-      <c r="AI1" s="56" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="2" spans="1:35">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="48" t="s">
-        <v>340</v>
-      </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="G2" s="47" t="s">
-        <v>339</v>
-      </c>
-      <c r="H2" s="22" t="s">
-        <v>342</v>
-      </c>
-      <c r="I2" s="1">
-        <v>1000</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="L2" t="s" s="0">
-        <v>319</v>
-      </c>
-      <c r="M2" s="38">
-        <f>ROUND(SUM(AA2+AB2+I2),2)</f>
-        <v>1000</v>
-      </c>
-      <c r="N2" s="38">
-        <f>ROUND(SUM(AA2+AB2+I2),2)</f>
-        <v>1000</v>
-      </c>
-      <c r="O2" s="1">
-        <v>88363222</v>
-      </c>
-      <c r="P2" s="53">
-        <v>0.18</v>
-      </c>
-      <c r="Q2" s="1">
-        <f>M2</f>
-        <v>1000</v>
-      </c>
-      <c r="R2" s="1">
-        <f>IF(OR($AE$1=1,$AE$1=4),ROUND((Q2*P2)/2,2),0)</f>
-        <v>90</v>
-      </c>
-      <c r="S2" s="1">
-        <f>IF($AE$1=1,ROUND(((Q2*P2)/2),2),0)</f>
-        <v>90</v>
-      </c>
-      <c r="T2" s="1">
-        <f>IF($AE$1=2,ROUND(((Q2*P2)),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="U2" s="1">
-        <f>IF($AE$1=4,ROUND(((Q2*P2)/2),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="V2" s="1">
-        <v>0</v>
-      </c>
-      <c r="W2" s="1">
-        <v>0</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="AA2" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="AB2" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="AC2" s="0">
-        <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)+R2+S2+T2+U2+W2),2)</f>
-        <v>1180</v>
-      </c>
-      <c r="AD2" t="s" s="0">
-        <v>337</v>
-      </c>
-      <c r="AE2" s="0">
-        <v>34</v>
-      </c>
-      <c r="AF2" t="s" s="0">
-        <v>345</v>
-      </c>
-      <c r="AG2" t="s" s="0">
-        <v>346</v>
-      </c>
-      <c r="AH2" s="53">
-        <v>0.01</v>
-      </c>
-      <c r="AI2" s="1">
-        <f>Q2*AH2</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:35">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="57" t="s">
-        <v>349</v>
-      </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="G3" s="47" t="s">
-        <v>339</v>
-      </c>
-      <c r="H3" s="22" t="s">
-        <v>342</v>
-      </c>
-      <c r="I3" s="1">
-        <f>AI2</f>
-        <v>10</v>
-      </c>
-      <c r="J3" s="14" t="s">
-        <v>303</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>207</v>
-      </c>
-      <c r="L3" s="1">
-        <v>1</v>
-      </c>
-      <c r="M3" s="38">
-        <f>M2*1%</f>
-        <v>10</v>
-      </c>
-      <c r="N3" s="38">
-        <f>M2*1%</f>
-        <v>10</v>
-      </c>
-      <c r="O3" s="1"/>
-      <c r="P3" s="53">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="1">
-        <v>0</v>
-      </c>
-      <c r="R3" s="1">
-        <f>IF(OR($AE$1=1,$AE$1=4),ROUND((Q3*P3)/2,2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="S3" s="1">
-        <f>IF($AE$1=1,ROUND(((Q3*P3)/2),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="T3" s="1">
-        <f>IF($AE$1=2,ROUND(((Q3*P3)),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="U3" s="1">
-        <f>IF($AE$1=4,ROUND(((Q3*P3)/2),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="V3" s="1">
-        <v>0</v>
-      </c>
-      <c r="W3" s="1">
-        <v>0</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="Z3" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="AA3" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="AB3" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="AC3" s="1">
-        <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)+R3+S3+T3+U3+W3),2)</f>
-        <v>10</v>
-      </c>
-      <c r="AD3" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="AE3" s="1"/>
-      <c r="AF3" s="1"/>
-      <c r="AG3" s="1"/>
-      <c r="AH3" s="1"/>
-      <c r="AI3" s="1"/>
-    </row>
-    <row r="4" spans="1:35">
-      <c r="I4" s="0">
-        <f>SUM(I2:I2)</f>
-        <v>1000</v>
-      </c>
-      <c r="M4" s="0">
-        <f>SUM(M2+R2+S2+T2+U2+W2)-M3</f>
-        <v>1170</v>
-      </c>
-      <c r="N4" s="0">
-        <f>SUM(N2+R2+S2+T2+U2+W2)-N3</f>
-        <v>1170</v>
-      </c>
-      <c r="Q4" s="0">
-        <f>SUM(Q2:Q2)</f>
-        <v>1000</v>
-      </c>
-      <c r="R4" s="0">
-        <f>SUM(R2:R2)</f>
-        <v>90</v>
-      </c>
-      <c r="S4" s="0">
-        <f>SUM(S2:S2)</f>
-        <v>90</v>
-      </c>
-      <c r="T4" s="0">
-        <f>SUM(T2:T2)</f>
-        <v>0</v>
-      </c>
-      <c r="U4" s="0">
-        <f>SUM(U2:U2)</f>
         <v>0</v>
       </c>
       <c r="AC4" s="0">
@@ -23187,10 +23221,10 @@
         <v>303</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>310</v>
+        <v>370</v>
       </c>
       <c r="AB2" t="s" s="0">
-        <v>310</v>
+        <v>370</v>
       </c>
       <c r="AC2" s="0">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
@@ -23264,10 +23298,10 @@
         <v>303</v>
       </c>
       <c r="AA3" t="s" s="0">
-        <v>310</v>
+        <v>370</v>
       </c>
       <c r="AB3" t="s" s="0">
-        <v>310</v>
+        <v>370</v>
       </c>
       <c r="AC3" s="0">
         <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>

</xml_diff>

<commit_message>
Fixes In The Cash Receipt screen Scenarios
Fixes In The Cash Receipt screen Scenarios
</commit_message>
<xml_diff>
--- a/testdata/Financials.xlsx
+++ b/testdata/Financials.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="136" activeTab="137"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="123" activeTab="125"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -131,37 +131,38 @@
     <sheet name="BPAdvJournalUSDNR" sheetId="150" r:id="rId122"/>
     <sheet name="JournalINRAdvNR" sheetId="144" r:id="rId123"/>
     <sheet name="BankReceipt" sheetId="35" r:id="rId124"/>
-    <sheet name="BankReceiptMulti" sheetId="37" r:id="rId125"/>
-    <sheet name="BRAdvUSDNR" sheetId="142" r:id="rId126"/>
-    <sheet name="BRAdvJournalUSDNR" sheetId="143" r:id="rId127"/>
-    <sheet name="BankReceiptUSD" sheetId="39" r:id="rId128"/>
-    <sheet name="BankReceiptMultiUSD" sheetId="40" r:id="rId129"/>
-    <sheet name="BankReceiptMulti (2)" sheetId="43" r:id="rId130"/>
-    <sheet name="BankReceiptMultiNewRef (2)" sheetId="44" r:id="rId131"/>
-    <sheet name="BankReceiptPDC" sheetId="56" r:id="rId132"/>
-    <sheet name="BankReceiptChargesUSD" sheetId="60" r:id="rId133"/>
-    <sheet name="BankReceiptCharges" sheetId="57" r:id="rId134"/>
-    <sheet name="BankPaymentChargesINR" sheetId="112" r:id="rId135"/>
-    <sheet name="BankPaymentCharges" sheetId="65" r:id="rId136"/>
-    <sheet name="BankPaymentExpGST" sheetId="63" r:id="rId137"/>
-    <sheet name="BankPaymentExpGSTTDS" sheetId="67" r:id="rId138"/>
-    <sheet name="BankPaymentExpUSD" sheetId="103" r:id="rId139"/>
-    <sheet name="BankPaymentExp" sheetId="62" r:id="rId140"/>
-    <sheet name="BankReceiptRevExp" sheetId="58" r:id="rId141"/>
-    <sheet name="BankPaymentExpTDS" sheetId="66" r:id="rId142"/>
-    <sheet name="BankPaymentPDC" sheetId="61" r:id="rId143"/>
-    <sheet name="BPAdvanceUSD" sheetId="161" r:id="rId144"/>
-    <sheet name="BPAdvance" sheetId="154" r:id="rId145"/>
-    <sheet name="BPJournalADV" sheetId="153" r:id="rId146"/>
-    <sheet name="TDS BPAdvance" sheetId="155" r:id="rId147"/>
-    <sheet name="TDS BPJournalADV" sheetId="156" r:id="rId148"/>
-    <sheet name="TDS BPAdvanceMulti" sheetId="157" r:id="rId149"/>
-    <sheet name="TDS BPJournalADVMulti" sheetId="158" r:id="rId150"/>
-    <sheet name="BPJournalADVINR" sheetId="159" r:id="rId151"/>
-    <sheet name="BPJournalADVUSD" sheetId="160" r:id="rId152"/>
-    <sheet name="BPMPMBADVNR" sheetId="162" r:id="rId153"/>
-    <sheet name="BPMPMBADVNRUSD" sheetId="163" r:id="rId154"/>
-    <sheet name="Sheet2" sheetId="146" r:id="rId155"/>
+    <sheet name="BankReceiptMultiCR" sheetId="168" r:id="rId125"/>
+    <sheet name="BankReceiptMulti" sheetId="37" r:id="rId126"/>
+    <sheet name="BRAdvUSDNR" sheetId="142" r:id="rId127"/>
+    <sheet name="BRAdvJournalUSDNR" sheetId="143" r:id="rId128"/>
+    <sheet name="BankReceiptUSD" sheetId="39" r:id="rId129"/>
+    <sheet name="BankReceiptMultiUSD" sheetId="40" r:id="rId130"/>
+    <sheet name="BankReceiptMulti (2)" sheetId="43" r:id="rId131"/>
+    <sheet name="BankReceiptMultiNewRef (2)" sheetId="44" r:id="rId132"/>
+    <sheet name="BankReceiptPDC" sheetId="56" r:id="rId133"/>
+    <sheet name="BankReceiptChargesUSD" sheetId="60" r:id="rId134"/>
+    <sheet name="BankReceiptCharges" sheetId="57" r:id="rId135"/>
+    <sheet name="BankPaymentChargesINR" sheetId="112" r:id="rId136"/>
+    <sheet name="BankPaymentCharges" sheetId="65" r:id="rId137"/>
+    <sheet name="BankPaymentExpGST" sheetId="63" r:id="rId138"/>
+    <sheet name="BankPaymentExpGSTTDS" sheetId="67" r:id="rId139"/>
+    <sheet name="BankPaymentExpUSD" sheetId="103" r:id="rId140"/>
+    <sheet name="BankPaymentExp" sheetId="62" r:id="rId141"/>
+    <sheet name="BankReceiptRevExp" sheetId="58" r:id="rId142"/>
+    <sheet name="BankPaymentExpTDS" sheetId="66" r:id="rId143"/>
+    <sheet name="BankPaymentPDC" sheetId="61" r:id="rId144"/>
+    <sheet name="BPAdvanceUSD" sheetId="161" r:id="rId145"/>
+    <sheet name="BPAdvance" sheetId="154" r:id="rId146"/>
+    <sheet name="BPJournalADV" sheetId="153" r:id="rId147"/>
+    <sheet name="TDS BPAdvance" sheetId="155" r:id="rId148"/>
+    <sheet name="TDS BPJournalADV" sheetId="156" r:id="rId149"/>
+    <sheet name="TDS BPAdvanceMulti" sheetId="157" r:id="rId150"/>
+    <sheet name="TDS BPJournalADVMulti" sheetId="158" r:id="rId151"/>
+    <sheet name="BPJournalADVINR" sheetId="159" r:id="rId152"/>
+    <sheet name="BPJournalADVUSD" sheetId="160" r:id="rId153"/>
+    <sheet name="BPMPMBADVNR" sheetId="162" r:id="rId154"/>
+    <sheet name="BPMPMBADVNRUSD" sheetId="163" r:id="rId155"/>
+    <sheet name="Sheet2" sheetId="146" r:id="rId156"/>
   </sheets>
   <calcPr calcId="124519"/>
   <extLst>
@@ -181,7 +182,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5626" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5591" uniqueCount="429">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -8393,6 +8394,300 @@
 
 <file path=xl/worksheets/sheet125.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AC4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="23.0"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.28515625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.85546875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="7.140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="14.5703125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="7.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="7.0"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="8.140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.5703125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="16.5703125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="5.5703125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="5.42578125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="5.0"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="6.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="8.42578125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="5.28515625"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="27" max="28" bestFit="true" customWidth="true" width="8.85546875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="20.0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:29">
+      <c r="A1" s="37" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" s="37" t="s">
+        <v>254</v>
+      </c>
+      <c r="C1" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="D1" s="37" t="s">
+        <v>255</v>
+      </c>
+      <c r="E1" s="37" t="s">
+        <v>279</v>
+      </c>
+      <c r="F1" s="37" t="s">
+        <v>256</v>
+      </c>
+      <c r="G1" s="37" t="s">
+        <v>257</v>
+      </c>
+      <c r="H1" s="37" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1" s="37" t="s">
+        <v>258</v>
+      </c>
+      <c r="J1" s="37" t="s">
+        <v>260</v>
+      </c>
+      <c r="K1" s="37" t="s">
+        <v>261</v>
+      </c>
+      <c r="L1" s="37" t="s">
+        <v>262</v>
+      </c>
+      <c r="M1" s="37" t="s">
+        <v>273</v>
+      </c>
+      <c r="N1" s="37" t="s">
+        <v>263</v>
+      </c>
+      <c r="O1" s="37" t="s">
+        <v>264</v>
+      </c>
+      <c r="P1" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="Q1" s="37" t="s">
+        <v>266</v>
+      </c>
+      <c r="R1" s="37" t="s">
+        <v>267</v>
+      </c>
+      <c r="S1" s="37" t="s">
+        <v>268</v>
+      </c>
+      <c r="T1" s="37" t="s">
+        <v>269</v>
+      </c>
+      <c r="U1" s="37" t="s">
+        <v>270</v>
+      </c>
+      <c r="V1" s="37" t="s">
+        <v>271</v>
+      </c>
+      <c r="W1" s="37" t="s">
+        <v>272</v>
+      </c>
+      <c r="X1" s="40" t="s">
+        <v>304</v>
+      </c>
+      <c r="Y1" s="40" t="s">
+        <v>204</v>
+      </c>
+      <c r="Z1" s="37" t="s">
+        <v>306</v>
+      </c>
+      <c r="AA1" s="40" t="s">
+        <v>307</v>
+      </c>
+      <c r="AB1" s="40" t="s">
+        <v>308</v>
+      </c>
+      <c r="AC1" s="40" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="48" t="s">
+        <v>318</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G2" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="H2" s="22" t="s">
+        <v>275</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>319</v>
+      </c>
+      <c r="M2" s="38">
+        <f>ROUND(SUM(AA2+AB2+I2),2)</f>
+        <v>0</v>
+      </c>
+      <c r="N2" s="38">
+        <f>AC2</f>
+        <v>0</v>
+      </c>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1">
+        <f>M2</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="AA2" t="s" s="0">
+        <v>428</v>
+      </c>
+      <c r="AB2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="AC2" s="0">
+        <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" s="1" customFormat="1">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G3" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>301</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="L3" t="s" s="0">
+        <v>319</v>
+      </c>
+      <c r="M3" s="38">
+        <f>ROUND(SUM(AA3+AB3+I3),2)</f>
+        <v>0</v>
+      </c>
+      <c r="N3" s="38">
+        <f>AC3</f>
+        <v>0</v>
+      </c>
+      <c r="Q3" s="1">
+        <f>M3</f>
+        <v>0</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="AA3" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="AB3" t="s" s="0">
+        <v>428</v>
+      </c>
+      <c r="AC3" s="0">
+        <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29">
+      <c r="I4" s="0">
+        <f>SUM(I2:I3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="0">
+        <f>SUM(M2:M3)</f>
+        <v>0</v>
+      </c>
+      <c r="N4" s="0">
+        <f>SUM(N2:N3)</f>
+        <v>0</v>
+      </c>
+      <c r="AC4" s="0">
+        <f>SUM(AC2:AC3)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet126.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet93"/>
   <dimension ref="A1:AC4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8583,10 +8878,10 @@
         <v>276</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>428</v>
+        <v>310</v>
       </c>
       <c r="AB2" t="s" s="0">
-        <v>428</v>
+        <v>310</v>
       </c>
       <c r="AC2" s="0">
         <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
@@ -8652,10 +8947,10 @@
         <v>276</v>
       </c>
       <c r="AA3" t="s" s="0">
-        <v>428</v>
+        <v>310</v>
       </c>
       <c r="AB3" t="s" s="0">
-        <v>428</v>
+        <v>310</v>
       </c>
       <c r="AC3" s="0">
         <f>ROUND(SUM((AA3*L3)+(AB3*L3)+(I3*L3)),2)</f>
@@ -8686,7 +8981,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet126.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet127.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AC3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -8917,7 +9212,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet127.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet128.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AE3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9085,7 +9380,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet128.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet129.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet94"/>
   <dimension ref="A1:AC3"/>
@@ -9317,7 +9612,56 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet129.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr codeName="Sheet13"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="25.5703125"/>
+    <col min="2" max="2" customWidth="true" width="15.140625"/>
+    <col min="3" max="3" customWidth="true" width="16.42578125"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet130.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet95"/>
   <dimension ref="A1:AC4"/>
@@ -9632,56 +9976,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr codeName="Sheet13"/>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" customWidth="true" width="25.5703125"/>
-    <col min="2" max="2" customWidth="true" width="15.140625"/>
-    <col min="3" max="3" customWidth="true" width="16.42578125"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="C2" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="C3" s="1">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet130.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet131.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet96"/>
   <dimension ref="A1:AC4"/>
@@ -9961,7 +10256,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet131.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet132.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet97"/>
   <dimension ref="A1:AC4"/>
@@ -10241,7 +10536,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet132.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet133.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet98"/>
   <dimension ref="A1:AD3"/>
@@ -10477,7 +10772,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet133.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet134.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet99"/>
   <dimension ref="A1:AD4"/>
@@ -10783,7 +11078,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet134.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet135.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet100"/>
   <dimension ref="A1:AD4"/>
@@ -11089,7 +11384,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet135.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet136.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet101"/>
   <dimension ref="A1:AD4"/>
@@ -11395,7 +11690,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet136.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet137.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet102"/>
   <dimension ref="A1:AD4"/>
@@ -11701,7 +11996,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet137.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet138.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet103"/>
   <dimension ref="A1:AG3"/>
@@ -11986,7 +12281,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet138.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet139.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet108"/>
   <dimension ref="A1:AL4"/>
@@ -12415,7 +12710,88 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet139.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr codeName="Sheet14"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="24.85546875"/>
+    <col min="2" max="2" customWidth="true" width="11.5703125"/>
+    <col min="3" max="3" customWidth="true" width="9.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.28515625"/>
+    <col min="5" max="5" customWidth="true" width="19.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.28515625"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="36" t="s">
+        <v>250</v>
+      </c>
+      <c r="E1" s="36" t="s">
+        <v>246</v>
+      </c>
+      <c r="F1" s="36" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" s="1">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="F2" s="0">
+        <f>ROUND(C2*E2,2)</f>
+        <v>847.48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C3" s="1">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>248</v>
+      </c>
+      <c r="F3" s="0">
+        <f>ROUND(C3*E3,2)</f>
+        <v>159.26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet140.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet104"/>
   <dimension ref="A1:AG3"/>
@@ -12700,88 +13076,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr codeName="Sheet14"/>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="24.85546875"/>
-    <col min="2" max="2" customWidth="true" width="11.5703125"/>
-    <col min="3" max="3" customWidth="true" width="9.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="19.28515625"/>
-    <col min="5" max="5" customWidth="true" width="19.28515625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.28515625"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="36" t="s">
-        <v>250</v>
-      </c>
-      <c r="E1" s="36" t="s">
-        <v>246</v>
-      </c>
-      <c r="F1" s="36" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="C2" s="1">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>249</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>251</v>
-      </c>
-      <c r="F2" s="0">
-        <f>ROUND(C2*E2,2)</f>
-        <v>847.48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="C3" s="1">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>252</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>248</v>
-      </c>
-      <c r="F3" s="0">
-        <f>ROUND(C3*E3,2)</f>
-        <v>159.26</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet140.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet141.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet105"/>
   <dimension ref="A1:AG3"/>
@@ -13066,7 +13361,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet141.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet142.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet106"/>
   <dimension ref="A1:AG4"/>
@@ -13454,7 +13749,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet142.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet143.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet107"/>
   <dimension ref="A1:AI4"/>
@@ -13849,7 +14144,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet143.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet144.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet109"/>
   <dimension ref="A1:AD3"/>
@@ -14077,237 +14372,6 @@
       </c>
       <c r="AD3" s="1" t="s">
         <v>337</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet144.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="29.0"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="10.85546875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="25.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="7.140625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="14.5703125"/>
-    <col min="8" max="8" customWidth="true" width="17.42578125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="12.140625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="7.0"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="8.140625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="15.5703125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="10.0"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="16.5703125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="5.5703125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="5.42578125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="5.0"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="6.85546875"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="8.42578125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="5.28515625"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="27" max="28" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="25.0"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:29">
-      <c r="A1" s="37" t="s">
-        <v>253</v>
-      </c>
-      <c r="B1" s="37" t="s">
-        <v>254</v>
-      </c>
-      <c r="C1" s="37" t="s">
-        <v>287</v>
-      </c>
-      <c r="D1" s="37" t="s">
-        <v>255</v>
-      </c>
-      <c r="E1" s="37" t="s">
-        <v>279</v>
-      </c>
-      <c r="F1" s="37" t="s">
-        <v>256</v>
-      </c>
-      <c r="G1" s="37" t="s">
-        <v>257</v>
-      </c>
-      <c r="H1" s="37" t="s">
-        <v>259</v>
-      </c>
-      <c r="I1" s="37" t="s">
-        <v>258</v>
-      </c>
-      <c r="J1" s="37" t="s">
-        <v>305</v>
-      </c>
-      <c r="K1" s="37" t="s">
-        <v>261</v>
-      </c>
-      <c r="L1" s="37" t="s">
-        <v>262</v>
-      </c>
-      <c r="M1" s="37" t="s">
-        <v>313</v>
-      </c>
-      <c r="N1" s="37" t="s">
-        <v>314</v>
-      </c>
-      <c r="O1" s="37" t="s">
-        <v>264</v>
-      </c>
-      <c r="P1" s="37" t="s">
-        <v>265</v>
-      </c>
-      <c r="Q1" s="37" t="s">
-        <v>266</v>
-      </c>
-      <c r="R1" s="37" t="s">
-        <v>267</v>
-      </c>
-      <c r="S1" s="37" t="s">
-        <v>268</v>
-      </c>
-      <c r="T1" s="37" t="s">
-        <v>269</v>
-      </c>
-      <c r="U1" s="46" t="s">
-        <v>270</v>
-      </c>
-      <c r="V1" s="46" t="s">
-        <v>271</v>
-      </c>
-      <c r="W1" s="46" t="s">
-        <v>272</v>
-      </c>
-      <c r="X1" s="40" t="s">
-        <v>304</v>
-      </c>
-      <c r="Y1" s="40" t="s">
-        <v>204</v>
-      </c>
-      <c r="Z1" s="37" t="s">
-        <v>306</v>
-      </c>
-      <c r="AA1" s="64" t="s">
-        <v>377</v>
-      </c>
-      <c r="AB1" s="64" t="s">
-        <v>378</v>
-      </c>
-      <c r="AC1" s="40" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="2" spans="1:29">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="75" t="s">
-        <v>397</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>399</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="G2" s="74" t="s">
-        <v>339</v>
-      </c>
-      <c r="H2" s="22" t="s">
-        <v>275</v>
-      </c>
-      <c r="I2" s="1">
-        <v>0</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="L2" t="s" s="0">
-        <v>369</v>
-      </c>
-      <c r="M2" s="38">
-        <f>ROUND(SUM(AA2+AB2+I2),2)</f>
-        <v>0</v>
-      </c>
-      <c r="N2" s="38">
-        <f>AC2</f>
-        <v>0</v>
-      </c>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1">
-        <f>M2</f>
-        <v>0</v>
-      </c>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
-      <c r="W2" s="1"/>
-      <c r="X2" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="AA2" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="AB2" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="AC2" s="0">
-        <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29">
-      <c r="M3" s="0">
-        <f>SUM(M2)</f>
-        <v>0</v>
-      </c>
-      <c r="N3" s="0">
-        <f>SUM(N2)</f>
-        <v>0</v>
-      </c>
-      <c r="Q3" s="0">
-        <f>SUM(Q2)</f>
-        <v>0</v>
-      </c>
-      <c r="AA3" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="AB3" s="0">
-        <v>0</v>
-      </c>
-      <c r="AC3" s="0">
-        <f>SUM(AC2)</f>
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -14444,14 +14508,14 @@
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="63" t="s">
-        <v>374</v>
+      <c r="B2" s="75" t="s">
+        <v>397</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>376</v>
+        <v>398</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>375</v>
+        <v>399</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>281</v>
@@ -14472,10 +14536,10 @@
         <v>276</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="L2" t="s" s="0">
-        <v>319</v>
+        <v>369</v>
       </c>
       <c r="M2" s="38">
         <f>ROUND(SUM(AA2+AB2+I2),2)</f>
@@ -14548,6 +14612,237 @@
 </file>
 
 <file path=xl/worksheets/sheet146.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AC3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="29.0"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="10.85546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="25.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="7.140625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="14.5703125"/>
+    <col min="8" max="8" customWidth="true" width="17.42578125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="12.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="7.0"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="8.140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="15.5703125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="16.5703125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="5.5703125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="5.42578125"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="5.0"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="6.85546875"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="8.42578125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="5.28515625"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="27" max="28" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="25.0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:29">
+      <c r="A1" s="37" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" s="37" t="s">
+        <v>254</v>
+      </c>
+      <c r="C1" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="D1" s="37" t="s">
+        <v>255</v>
+      </c>
+      <c r="E1" s="37" t="s">
+        <v>279</v>
+      </c>
+      <c r="F1" s="37" t="s">
+        <v>256</v>
+      </c>
+      <c r="G1" s="37" t="s">
+        <v>257</v>
+      </c>
+      <c r="H1" s="37" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1" s="37" t="s">
+        <v>258</v>
+      </c>
+      <c r="J1" s="37" t="s">
+        <v>305</v>
+      </c>
+      <c r="K1" s="37" t="s">
+        <v>261</v>
+      </c>
+      <c r="L1" s="37" t="s">
+        <v>262</v>
+      </c>
+      <c r="M1" s="37" t="s">
+        <v>313</v>
+      </c>
+      <c r="N1" s="37" t="s">
+        <v>314</v>
+      </c>
+      <c r="O1" s="37" t="s">
+        <v>264</v>
+      </c>
+      <c r="P1" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="Q1" s="37" t="s">
+        <v>266</v>
+      </c>
+      <c r="R1" s="37" t="s">
+        <v>267</v>
+      </c>
+      <c r="S1" s="37" t="s">
+        <v>268</v>
+      </c>
+      <c r="T1" s="37" t="s">
+        <v>269</v>
+      </c>
+      <c r="U1" s="46" t="s">
+        <v>270</v>
+      </c>
+      <c r="V1" s="46" t="s">
+        <v>271</v>
+      </c>
+      <c r="W1" s="46" t="s">
+        <v>272</v>
+      </c>
+      <c r="X1" s="40" t="s">
+        <v>304</v>
+      </c>
+      <c r="Y1" s="40" t="s">
+        <v>204</v>
+      </c>
+      <c r="Z1" s="37" t="s">
+        <v>306</v>
+      </c>
+      <c r="AA1" s="64" t="s">
+        <v>377</v>
+      </c>
+      <c r="AB1" s="64" t="s">
+        <v>378</v>
+      </c>
+      <c r="AC1" s="40" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="63" t="s">
+        <v>374</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G2" s="74" t="s">
+        <v>339</v>
+      </c>
+      <c r="H2" s="22" t="s">
+        <v>275</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>319</v>
+      </c>
+      <c r="M2" s="38">
+        <f>ROUND(SUM(AA2+AB2+I2),2)</f>
+        <v>0</v>
+      </c>
+      <c r="N2" s="38">
+        <f>AC2</f>
+        <v>0</v>
+      </c>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1">
+        <f>M2</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="AA2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="AB2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="AC2" s="0">
+        <f>ROUND(SUM((AA2*L2)+(AB2*L2)+(I2*L2)),2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29">
+      <c r="M3" s="0">
+        <f>SUM(M2)</f>
+        <v>0</v>
+      </c>
+      <c r="N3" s="0">
+        <f>SUM(N2)</f>
+        <v>0</v>
+      </c>
+      <c r="Q3" s="0">
+        <f>SUM(Q2)</f>
+        <v>0</v>
+      </c>
+      <c r="AA3" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="AB3" s="0">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="0">
+        <f>SUM(AC2)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet147.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AE3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -14711,7 +15006,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet147.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet148.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AH4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15045,7 +15340,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet148.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet149.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AE9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15256,7 +15551,56 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet149.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr codeName="Sheet15"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="21.42578125"/>
+    <col min="2" max="2" customWidth="true" width="11.5703125"/>
+    <col min="3" max="3" customWidth="true" width="9.0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet150.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AH6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15804,56 +16148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr codeName="Sheet15"/>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" customWidth="true" width="21.42578125"/>
-    <col min="2" max="2" customWidth="true" width="11.5703125"/>
-    <col min="3" max="3" customWidth="true" width="9.0"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="C2" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="C3" s="1">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet150.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet151.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AE11"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -16150,170 +16445,6 @@
       </c>
     </row>
     <row r="11" spans="1:31" ht="9" customHeight="1"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet151.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="23.0"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="28.7109375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="33.42578125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="28.7109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="18.42578125"/>
-    <col min="7" max="8" customWidth="true" width="18.42578125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="14.5703125"/>
-    <col min="10" max="10" customWidth="true" width="17.42578125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="21.5703125"/>
-    <col min="13" max="13" customWidth="true" width="21.5703125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="16.0"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="16.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="16.5703125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="15.0"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="20.0"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:31">
-      <c r="A1" s="56" t="s">
-        <v>253</v>
-      </c>
-      <c r="B1" s="56" t="s">
-        <v>183</v>
-      </c>
-      <c r="C1" s="56" t="s">
-        <v>352</v>
-      </c>
-      <c r="D1" s="56" t="s">
-        <v>254</v>
-      </c>
-      <c r="E1" s="56" t="s">
-        <v>353</v>
-      </c>
-      <c r="F1" s="56" t="s">
-        <v>257</v>
-      </c>
-      <c r="G1" s="56" t="s">
-        <v>357</v>
-      </c>
-      <c r="H1" s="56" t="s">
-        <v>358</v>
-      </c>
-      <c r="I1" s="56" t="s">
-        <v>354</v>
-      </c>
-      <c r="J1" s="56" t="s">
-        <v>355</v>
-      </c>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
-      <c r="P1" s="37"/>
-      <c r="Q1" s="37"/>
-      <c r="R1" s="37"/>
-      <c r="S1" s="37"/>
-      <c r="T1" s="37"/>
-      <c r="U1" s="37"/>
-      <c r="V1" s="37"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="46"/>
-      <c r="Y1" s="46"/>
-      <c r="Z1" s="40"/>
-      <c r="AA1" s="40"/>
-      <c r="AB1" s="37"/>
-      <c r="AC1" s="40"/>
-      <c r="AD1" s="40"/>
-      <c r="AE1" s="40"/>
-    </row>
-    <row r="2" spans="1:31">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="58" t="s">
-        <v>191</v>
-      </c>
-      <c r="C2" s="1">
-        <v>2000000099</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="I2" s="47">
-        <f>ROUND(SUM(G2+H2),2)</f>
-        <v>0</v>
-      </c>
-      <c r="J2" s="59">
-        <v>0</v>
-      </c>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="O2" s="38"/>
-      <c r="P2" s="38"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
-      <c r="W2" s="1"/>
-      <c r="X2" s="1"/>
-      <c r="Y2" s="1"/>
-      <c r="Z2" s="1"/>
-      <c r="AA2" s="1"/>
-      <c r="AB2" s="1"/>
-    </row>
-    <row r="3" spans="1:31">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="58" t="s">
-        <v>191</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1001002003</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="H3" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="I3" s="59">
-        <v>0</v>
-      </c>
-      <c r="J3" s="59">
-        <f>ROUND(SUM(G3+H3),2)</f>
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -16381,9 +16512,7 @@
       <c r="J1" s="56" t="s">
         <v>355</v>
       </c>
-      <c r="K1" t="s" s="0">
-        <v>369</v>
-      </c>
+      <c r="K1" s="37"/>
       <c r="L1" s="37"/>
       <c r="M1" s="37"/>
       <c r="N1" s="37"/>
@@ -16413,10 +16542,10 @@
         <v>191</v>
       </c>
       <c r="C2" s="1">
-        <v>2000000118</v>
+        <v>2000000099</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>397</v>
+        <v>374</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -16427,8 +16556,8 @@
         <v>310</v>
       </c>
       <c r="I2" s="47">
-        <f>ROUND(SUM(G2+H2)*K1,2)</f>
-        <v>15937.5</v>
+        <f>ROUND(SUM(G2+H2),2)</f>
+        <v>0</v>
       </c>
       <c r="J2" s="59">
         <v>0</v>
@@ -16459,10 +16588,10 @@
         <v>191</v>
       </c>
       <c r="C3" s="1">
-        <v>1001002001</v>
+        <v>1001002003</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -16476,8 +16605,8 @@
         <v>0</v>
       </c>
       <c r="J3" s="59">
-        <f>ROUND(SUM(G3+H3)*K1,2)</f>
-        <v>15937.5</v>
+        <f>ROUND(SUM(G3+H3),2)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -16487,6 +16616,172 @@
 </file>
 
 <file path=xl/worksheets/sheet153.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AE3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="23.0"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="28.7109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="33.42578125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="28.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="18.42578125"/>
+    <col min="7" max="8" customWidth="true" width="18.42578125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="14.5703125"/>
+    <col min="10" max="10" customWidth="true" width="17.42578125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="21.5703125"/>
+    <col min="13" max="13" customWidth="true" width="21.5703125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="16.0"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="16.7109375"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="16.5703125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="20.0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31">
+      <c r="A1" s="56" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" s="56" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1" s="56" t="s">
+        <v>352</v>
+      </c>
+      <c r="D1" s="56" t="s">
+        <v>254</v>
+      </c>
+      <c r="E1" s="56" t="s">
+        <v>353</v>
+      </c>
+      <c r="F1" s="56" t="s">
+        <v>257</v>
+      </c>
+      <c r="G1" s="56" t="s">
+        <v>357</v>
+      </c>
+      <c r="H1" s="56" t="s">
+        <v>358</v>
+      </c>
+      <c r="I1" s="56" t="s">
+        <v>354</v>
+      </c>
+      <c r="J1" s="56" t="s">
+        <v>355</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>369</v>
+      </c>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="37"/>
+      <c r="T1" s="37"/>
+      <c r="U1" s="37"/>
+      <c r="V1" s="37"/>
+      <c r="W1" s="46"/>
+      <c r="X1" s="46"/>
+      <c r="Y1" s="46"/>
+      <c r="Z1" s="40"/>
+      <c r="AA1" s="40"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="40"/>
+      <c r="AD1" s="40"/>
+      <c r="AE1" s="40"/>
+    </row>
+    <row r="2" spans="1:31">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="58" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2000000118</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="I2" s="47">
+        <f>ROUND(SUM(G2+H2)*K1,2)</f>
+        <v>15937.5</v>
+      </c>
+      <c r="J2" s="59">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="O2" s="38"/>
+      <c r="P2" s="38"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+    </row>
+    <row r="3" spans="1:31">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="58" t="s">
+        <v>191</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1001002001</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="I3" s="59">
+        <v>0</v>
+      </c>
+      <c r="J3" s="59">
+        <f>ROUND(SUM(G3+H3)*K1,2)</f>
+        <v>15937.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet154.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AI4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -16885,7 +17180,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet154.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet155.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AI4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -17284,7 +17579,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet155.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet156.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -24444,7 +24739,7 @@
         <v>303</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>310</v>
+        <v>426</v>
       </c>
       <c r="AB2" t="s" s="0">
         <v>310</v>
@@ -37148,8 +37443,8 @@
       <c r="G2" t="s" s="0">
         <v>310</v>
       </c>
-      <c r="H2" s="0">
-        <v>0</v>
+      <c r="H2" t="s" s="0">
+        <v>310</v>
       </c>
       <c r="I2" s="47">
         <f>ROUND(SUM(G2+H2),2)</f>
@@ -37194,8 +37489,8 @@
       <c r="G3" t="s" s="0">
         <v>310</v>
       </c>
-      <c r="H3" s="0">
-        <v>0</v>
+      <c r="H3" t="s" s="0">
+        <v>310</v>
       </c>
       <c r="I3" s="59">
         <v>0</v>

</xml_diff>